<commit_message>
Commit for Day 5 and Day 6 of project. Dashboard and Report completed.
</commit_message>
<xml_diff>
--- a/Data Analysis Project/project/reports/Dashboard.xlsx
+++ b/Data Analysis Project/project/reports/Dashboard.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_RushilJivan_2026\Data Analysis Project\project\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{71CF6F8D-8E5A-4E66-9817-4BBE9AA6BAF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1331F6F3-2728-4C52-8D12-4017D03B83AD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="clean_sales" sheetId="5" r:id="rId1"/>
@@ -28,7 +28,7 @@
   </definedNames>
   <calcPr calcId="191029"/>
   <pivotCaches>
-    <pivotCache cacheId="0" r:id="rId4"/>
+    <pivotCache cacheId="1" r:id="rId4"/>
   </pivotCaches>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{BBE1A952-AA13-448e-AADC-164F8A28A991}">
@@ -71,7 +71,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="270" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="278" uniqueCount="39">
   <si>
     <t>transaction_id</t>
   </si>
@@ -1620,7 +1620,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$B$44:$B$45</c:f>
+              <c:f>Pivot_Tables!$B$54:$B$55</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1643,7 +1643,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$46:$A$50</c:f>
+              <c:f>Pivot_Tables!$A$56:$A$60</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1663,7 +1663,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$B$46:$B$50</c:f>
+              <c:f>Pivot_Tables!$B$56:$B$60</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1690,7 +1690,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$C$44:$C$45</c:f>
+              <c:f>Pivot_Tables!$C$54:$C$55</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1713,7 +1713,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$46:$A$50</c:f>
+              <c:f>Pivot_Tables!$A$56:$A$60</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1733,7 +1733,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$C$46:$C$50</c:f>
+              <c:f>Pivot_Tables!$C$56:$C$60</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1754,7 +1754,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000005-4DFF-42FD-9CF6-881540224D51}"/>
+              <c16:uniqueId val="{0000000F-FC4F-4877-B825-4B311FCC7DEE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1763,7 +1763,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$D$44:$D$45</c:f>
+              <c:f>Pivot_Tables!$D$54:$D$55</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1784,7 +1784,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$46:$A$50</c:f>
+              <c:f>Pivot_Tables!$A$56:$A$60</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1804,7 +1804,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$D$46:$D$50</c:f>
+              <c:f>Pivot_Tables!$D$56:$D$60</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1825,7 +1825,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000006-4DFF-42FD-9CF6-881540224D51}"/>
+              <c16:uniqueId val="{00000010-FC4F-4877-B825-4B311FCC7DEE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1834,7 +1834,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$E$44:$E$45</c:f>
+              <c:f>Pivot_Tables!$E$54:$E$55</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1857,7 +1857,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$46:$A$50</c:f>
+              <c:f>Pivot_Tables!$A$56:$A$60</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1877,7 +1877,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$E$46:$E$50</c:f>
+              <c:f>Pivot_Tables!$E$56:$E$60</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1898,7 +1898,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000007-4DFF-42FD-9CF6-881540224D51}"/>
+              <c16:uniqueId val="{00000011-FC4F-4877-B825-4B311FCC7DEE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1907,7 +1907,7 @@
           <c:order val="4"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$F$44:$F$45</c:f>
+              <c:f>Pivot_Tables!$F$54:$F$55</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -1930,7 +1930,7 @@
           <c:invertIfNegative val="0"/>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$46:$A$50</c:f>
+              <c:f>Pivot_Tables!$A$56:$A$60</c:f>
               <c:strCache>
                 <c:ptCount val="4"/>
                 <c:pt idx="0">
@@ -1950,7 +1950,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$F$46:$F$50</c:f>
+              <c:f>Pivot_Tables!$F$56:$F$60</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="4"/>
@@ -1971,7 +1971,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000009-4DFF-42FD-9CF6-881540224D51}"/>
+              <c16:uniqueId val="{00000012-FC4F-4877-B825-4B311FCC7DEE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2193,14 +2193,14 @@
   <c:roundedCorners val="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" Requires="c14">
-      <c14:style val="107"/>
+      <c14:style val="102"/>
     </mc:Choice>
     <mc:Fallback>
-      <c:style val="7"/>
+      <c:style val="2"/>
     </mc:Fallback>
   </mc:AlternateContent>
   <c:pivotSource>
-    <c:name>[Dashboard.xlsx]Pivot_Tables!Salesperson Performance</c:name>
+    <c:name>[Dashboard.xlsx]Pivot_Tables!Salesperson Performance Monthly</c:name>
     <c:fmtId val="3"/>
   </c:pivotSource>
   <c:chart>
@@ -2210,7 +2210,7 @@
         <c:idx val="0"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent5"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -2222,11 +2222,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2278,7 +2278,7 @@
         <c:idx val="1"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent5"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -2290,11 +2290,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2346,7 +2346,7 @@
         <c:idx val="2"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent5"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -2358,11 +2358,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2414,7 +2414,7 @@
         <c:idx val="3"/>
         <c:spPr>
           <a:solidFill>
-            <a:schemeClr val="accent5"/>
+            <a:schemeClr val="accent1"/>
           </a:solidFill>
           <a:ln>
             <a:noFill/>
@@ -2426,11 +2426,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2483,7 +2483,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -2494,15 +2494,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:tint val="58000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:tint val="58000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2552,7 +2548,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -2563,15 +2559,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:tint val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent3"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:tint val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent3"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2621,7 +2613,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -2632,15 +2624,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent5"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent5"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2690,7 +2678,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -2701,14 +2689,14 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="58000"/>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
             </a:ln>
@@ -2759,9 +2747,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:tint val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -2772,15 +2758,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:tint val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent3"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:tint val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent3"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2836,9 +2818,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -2849,14 +2829,14 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="58000"/>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
             </a:ln>
@@ -2913,9 +2893,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -2926,15 +2904,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent5"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent5"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -2990,9 +2964,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -3003,14 +2975,14 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="58000"/>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
             </a:ln>
@@ -3067,9 +3039,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -3080,14 +3050,14 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="58000"/>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
             </a:ln>
@@ -3144,9 +3114,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -3157,14 +3125,14 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="58000"/>
+              <a:schemeClr val="accent1">
+                <a:lumMod val="60000"/>
               </a:schemeClr>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="58000"/>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
             </a:ln>
@@ -3221,9 +3189,7 @@
         <c:spPr>
           <a:ln w="28575" cap="rnd">
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:round/>
           </a:ln>
@@ -3234,15 +3200,11 @@
           <c:size val="5"/>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5">
-                <a:shade val="86000"/>
-              </a:schemeClr>
+              <a:schemeClr val="accent5"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent5"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -3296,22 +3258,22 @@
       <c:pivotFmt>
         <c:idx val="15"/>
         <c:spPr>
-          <a:ln w="28575" cap="rnd">
-            <a:solidFill>
-              <a:schemeClr val="accent5"/>
-            </a:solidFill>
-            <a:round/>
+          <a:solidFill>
+            <a:schemeClr val="accent1"/>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
           </a:ln>
           <a:effectLst/>
         </c:spPr>
         <c:marker>
           <c:spPr>
             <a:solidFill>
-              <a:schemeClr val="accent5"/>
+              <a:schemeClr val="accent1"/>
             </a:solidFill>
             <a:ln w="9525">
               <a:solidFill>
-                <a:schemeClr val="accent5"/>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
             </a:ln>
             <a:effectLst/>
@@ -3368,7 +3330,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$B$54:$B$57</c:f>
+              <c:f>Pivot_Tables!$B$64:$B$67</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3380,9 +3342,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:tint val="58000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3393,15 +3353,11 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:tint val="58000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent1"/>
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:tint val="58000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent1"/>
                 </a:solidFill>
               </a:ln>
               <a:effectLst/>
@@ -3463,7 +3419,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$58:$A$63</c:f>
+              <c:f>Pivot_Tables!$A$68:$A$73</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3486,7 +3442,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$B$58:$B$63</c:f>
+              <c:f>Pivot_Tables!$B$68:$B$73</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3517,7 +3473,7 @@
           <c:order val="1"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$C$54:$C$57</c:f>
+              <c:f>Pivot_Tables!$C$64:$C$67</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3529,9 +3485,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:tint val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent3"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3542,15 +3496,11 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:tint val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent3"/>
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:tint val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent3"/>
                 </a:solidFill>
               </a:ln>
               <a:effectLst/>
@@ -3563,15 +3513,11 @@
               <c:size val="5"/>
               <c:spPr>
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:tint val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent3"/>
                 </a:solidFill>
                 <a:ln w="9525">
                   <a:solidFill>
-                    <a:schemeClr val="accent5">
-                      <a:tint val="86000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="accent3"/>
                   </a:solidFill>
                 </a:ln>
                 <a:effectLst/>
@@ -3581,14 +3527,17 @@
             <c:spPr>
               <a:ln w="28575" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:tint val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent3"/>
                 </a:solidFill>
                 <a:round/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-BE35-4292-88E3-9653B484C7BF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:dLbl>
@@ -3608,6 +3557,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-BE35-4292-88E3-9653B484C7BF}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:numFmt formatCode="&quot;R&quot;#,##0.00" sourceLinked="0"/>
@@ -3665,7 +3617,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$58:$A$63</c:f>
+              <c:f>Pivot_Tables!$A$68:$A$73</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3688,7 +3640,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$C$58:$C$63</c:f>
+              <c:f>Pivot_Tables!$C$68:$C$73</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3722,7 +3674,7 @@
           <c:order val="2"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$D$54:$D$57</c:f>
+              <c:f>Pivot_Tables!$D$64:$D$67</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3734,9 +3686,7 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent5"/>
               </a:solidFill>
               <a:round/>
             </a:ln>
@@ -3747,15 +3697,11 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="86000"/>
-                </a:schemeClr>
+                <a:schemeClr val="accent5"/>
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent5"/>
                 </a:solidFill>
               </a:ln>
               <a:effectLst/>
@@ -3768,15 +3714,11 @@
               <c:size val="5"/>
               <c:spPr>
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent5"/>
                 </a:solidFill>
                 <a:ln w="9525">
                   <a:solidFill>
-                    <a:schemeClr val="accent5">
-                      <a:shade val="86000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="accent5"/>
                   </a:solidFill>
                 </a:ln>
                 <a:effectLst/>
@@ -3786,14 +3728,17 @@
             <c:spPr>
               <a:ln w="28575" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent5"/>
                 </a:solidFill>
                 <a:round/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000003-BE35-4292-88E3-9653B484C7BF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dPt>
             <c:idx val="2"/>
@@ -3802,15 +3747,11 @@
               <c:size val="5"/>
               <c:spPr>
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent5"/>
                 </a:solidFill>
                 <a:ln w="9525">
                   <a:solidFill>
-                    <a:schemeClr val="accent5">
-                      <a:shade val="86000"/>
-                    </a:schemeClr>
+                    <a:schemeClr val="accent5"/>
                   </a:solidFill>
                 </a:ln>
                 <a:effectLst/>
@@ -3820,14 +3761,17 @@
             <c:spPr>
               <a:ln w="28575" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="86000"/>
-                  </a:schemeClr>
+                  <a:schemeClr val="accent5"/>
                 </a:solidFill>
                 <a:round/>
               </a:ln>
               <a:effectLst/>
             </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000005-BE35-4292-88E3-9653B484C7BF}"/>
+              </c:ext>
+            </c:extLst>
           </c:dPt>
           <c:dLbls>
             <c:dLbl>
@@ -3847,6 +3791,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000003-BE35-4292-88E3-9653B484C7BF}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:dLbl>
@@ -3866,6 +3813,9 @@
               <c:showBubbleSize val="0"/>
               <c:extLst>
                 <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000005-BE35-4292-88E3-9653B484C7BF}"/>
+                </c:ext>
               </c:extLst>
             </c:dLbl>
             <c:numFmt formatCode="&quot;R&quot;#,##0.00" sourceLinked="0"/>
@@ -3923,7 +3873,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$58:$A$63</c:f>
+              <c:f>Pivot_Tables!$A$68:$A$73</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -3946,7 +3896,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$D$58:$D$63</c:f>
+              <c:f>Pivot_Tables!$D$68:$D$73</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -3977,7 +3927,7 @@
           <c:order val="3"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$E$54:$E$57</c:f>
+              <c:f>Pivot_Tables!$E$64:$E$67</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -3989,8 +3939,8 @@
           <c:spPr>
             <a:ln w="28575" cap="rnd">
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="58000"/>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:round/>
@@ -4002,14 +3952,14 @@
             <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
-                <a:schemeClr val="accent5">
-                  <a:shade val="58000"/>
+                <a:schemeClr val="accent1">
+                  <a:lumMod val="60000"/>
                 </a:schemeClr>
               </a:solidFill>
               <a:ln w="9525">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
               </a:ln>
@@ -4023,14 +3973,14 @@
               <c:size val="5"/>
               <c:spPr>
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:ln w="9525">
                   <a:solidFill>
-                    <a:schemeClr val="accent5">
-                      <a:shade val="58000"/>
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="60000"/>
                     </a:schemeClr>
                   </a:solidFill>
                 </a:ln>
@@ -4041,8 +3991,8 @@
             <c:spPr>
               <a:ln w="28575" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:round/>
@@ -4057,14 +4007,14 @@
               <c:size val="5"/>
               <c:spPr>
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:ln w="9525">
                   <a:solidFill>
-                    <a:schemeClr val="accent5">
-                      <a:shade val="58000"/>
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="60000"/>
                     </a:schemeClr>
                   </a:solidFill>
                 </a:ln>
@@ -4075,8 +4025,8 @@
             <c:spPr>
               <a:ln w="28575" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:round/>
@@ -4091,14 +4041,14 @@
               <c:size val="5"/>
               <c:spPr>
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:ln w="9525">
                   <a:solidFill>
-                    <a:schemeClr val="accent5">
-                      <a:shade val="58000"/>
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="60000"/>
                     </a:schemeClr>
                   </a:solidFill>
                 </a:ln>
@@ -4109,8 +4059,8 @@
             <c:spPr>
               <a:ln w="28575" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:round/>
@@ -4125,14 +4075,14 @@
               <c:size val="5"/>
               <c:spPr>
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:ln w="9525">
                   <a:solidFill>
-                    <a:schemeClr val="accent5">
-                      <a:shade val="58000"/>
+                    <a:schemeClr val="accent1">
+                      <a:lumMod val="60000"/>
                     </a:schemeClr>
                   </a:solidFill>
                 </a:ln>
@@ -4143,8 +4093,8 @@
             <c:spPr>
               <a:ln w="28575" cap="rnd">
                 <a:solidFill>
-                  <a:schemeClr val="accent5">
-                    <a:shade val="58000"/>
+                  <a:schemeClr val="accent1">
+                    <a:lumMod val="60000"/>
                   </a:schemeClr>
                 </a:solidFill>
                 <a:round/>
@@ -4284,7 +4234,7 @@
           </c:dLbls>
           <c:cat>
             <c:strRef>
-              <c:f>Pivot_Tables!$A$58:$A$63</c:f>
+              <c:f>Pivot_Tables!$A$68:$A$73</c:f>
               <c:strCache>
                 <c:ptCount val="5"/>
                 <c:pt idx="0">
@@ -4307,7 +4257,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$E$58:$E$63</c:f>
+              <c:f>Pivot_Tables!$E$68:$E$73</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -4332,7 +4282,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000011-1E96-4179-B2E6-ECA064132FD3}"/>
+              <c16:uniqueId val="{00000010-BE35-4292-88E3-9653B484C7BF}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4766,7 +4716,7 @@
           <c:order val="0"/>
           <c:tx>
             <c:strRef>
-              <c:f>Pivot_Tables!$B$29</c:f>
+              <c:f>Pivot_Tables!$B$39</c:f>
               <c:strCache>
                 <c:ptCount val="1"/>
                 <c:pt idx="0">
@@ -4934,7 +4884,7 @@
           </c:dLbls>
           <c:cat>
             <c:multiLvlStrRef>
-              <c:f>Pivot_Tables!$A$30:$A$40</c:f>
+              <c:f>Pivot_Tables!$A$40:$A$50</c:f>
               <c:multiLvlStrCache>
                 <c:ptCount val="5"/>
                 <c:lvl>
@@ -4976,7 +4926,7 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Pivot_Tables!$B$30:$B$40</c:f>
+              <c:f>Pivot_Tables!$B$40:$B$50</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="5"/>
@@ -5141,8 +5091,39 @@
 </file>
 
 <file path=xl/charts/colors4.xml><?xml version="1.0" encoding="utf-8"?>
-<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="withinLinearReversed" id="25">
+<cs:colorStyle xmlns:cs="http://schemas.microsoft.com/office/drawing/2012/chartStyle" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" meth="cycle" id="11">
+  <a:schemeClr val="accent1"/>
+  <a:schemeClr val="accent3"/>
   <a:schemeClr val="accent5"/>
+  <cs:variation/>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+    <a:lumOff val="20000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="80000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="60000"/>
+    <a:lumOff val="40000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+    <a:lumOff val="30000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="70000"/>
+  </cs:variation>
+  <cs:variation>
+    <a:lumMod val="50000"/>
+    <a:lumOff val="50000"/>
+  </cs:variation>
 </cs:colorStyle>
 </file>
 
@@ -10276,8 +10257,657 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2EBA4ED6-0263-4163-B60D-94E9DAE81843}" name="Product Category Distribution" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="27">
-  <location ref="A29:B40" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A92E6C64-2F9D-443D-AE81-1304DED4A368}" name="Saleperson Performance" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="3" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A29:B35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="14">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{77BF86ED-9B5C-443E-BA35-5E459117CD3F}" name="Top Performing Products" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+  <location ref="A10:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="368">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+        <item sd="0" x="14"/>
+        <item sd="0" x="15"/>
+        <item sd="0" x="16"/>
+        <item sd="0" x="17"/>
+        <item sd="0" x="18"/>
+        <item sd="0" x="19"/>
+        <item sd="0" x="20"/>
+        <item sd="0" x="21"/>
+        <item sd="0" x="22"/>
+        <item sd="0" x="23"/>
+        <item sd="0" x="24"/>
+        <item sd="0" x="25"/>
+        <item sd="0" x="26"/>
+        <item sd="0" x="27"/>
+        <item sd="0" x="28"/>
+        <item sd="0" x="29"/>
+        <item sd="0" x="30"/>
+        <item sd="0" x="31"/>
+        <item sd="0" x="32"/>
+        <item sd="0" x="33"/>
+        <item sd="0" x="34"/>
+        <item sd="0" x="35"/>
+        <item sd="0" x="36"/>
+        <item sd="0" x="37"/>
+        <item sd="0" x="38"/>
+        <item sd="0" x="39"/>
+        <item sd="0" x="40"/>
+        <item sd="0" x="41"/>
+        <item sd="0" x="42"/>
+        <item sd="0" x="43"/>
+        <item sd="0" x="44"/>
+        <item sd="0" x="45"/>
+        <item sd="0" x="46"/>
+        <item sd="0" x="47"/>
+        <item sd="0" x="48"/>
+        <item sd="0" x="49"/>
+        <item sd="0" x="50"/>
+        <item sd="0" x="51"/>
+        <item sd="0" x="52"/>
+        <item sd="0" x="53"/>
+        <item sd="0" x="54"/>
+        <item sd="0" x="55"/>
+        <item sd="0" x="56"/>
+        <item sd="0" x="57"/>
+        <item sd="0" x="58"/>
+        <item sd="0" x="59"/>
+        <item sd="0" x="60"/>
+        <item sd="0" x="61"/>
+        <item sd="0" x="62"/>
+        <item sd="0" x="63"/>
+        <item sd="0" x="64"/>
+        <item sd="0" x="65"/>
+        <item sd="0" x="66"/>
+        <item sd="0" x="67"/>
+        <item sd="0" x="68"/>
+        <item sd="0" x="69"/>
+        <item sd="0" x="70"/>
+        <item sd="0" x="71"/>
+        <item sd="0" x="72"/>
+        <item sd="0" x="73"/>
+        <item sd="0" x="74"/>
+        <item sd="0" x="75"/>
+        <item sd="0" x="76"/>
+        <item sd="0" x="77"/>
+        <item sd="0" x="78"/>
+        <item sd="0" x="79"/>
+        <item sd="0" x="80"/>
+        <item sd="0" x="81"/>
+        <item sd="0" x="82"/>
+        <item sd="0" x="83"/>
+        <item sd="0" x="84"/>
+        <item sd="0" x="85"/>
+        <item sd="0" x="86"/>
+        <item sd="0" x="87"/>
+        <item sd="0" x="88"/>
+        <item sd="0" x="89"/>
+        <item sd="0" x="90"/>
+        <item sd="0" x="91"/>
+        <item sd="0" x="92"/>
+        <item sd="0" x="93"/>
+        <item sd="0" x="94"/>
+        <item sd="0" x="95"/>
+        <item sd="0" x="96"/>
+        <item sd="0" x="97"/>
+        <item sd="0" x="98"/>
+        <item sd="0" x="99"/>
+        <item sd="0" x="100"/>
+        <item sd="0" x="101"/>
+        <item sd="0" x="102"/>
+        <item sd="0" x="103"/>
+        <item sd="0" x="104"/>
+        <item sd="0" x="105"/>
+        <item sd="0" x="106"/>
+        <item sd="0" x="107"/>
+        <item sd="0" x="108"/>
+        <item sd="0" x="109"/>
+        <item sd="0" x="110"/>
+        <item sd="0" x="111"/>
+        <item sd="0" x="112"/>
+        <item sd="0" x="113"/>
+        <item sd="0" x="114"/>
+        <item sd="0" x="115"/>
+        <item sd="0" x="116"/>
+        <item sd="0" x="117"/>
+        <item sd="0" x="118"/>
+        <item sd="0" x="119"/>
+        <item sd="0" x="120"/>
+        <item sd="0" x="121"/>
+        <item sd="0" x="122"/>
+        <item sd="0" x="123"/>
+        <item sd="0" x="124"/>
+        <item sd="0" x="125"/>
+        <item sd="0" x="126"/>
+        <item sd="0" x="127"/>
+        <item sd="0" x="128"/>
+        <item sd="0" x="129"/>
+        <item sd="0" x="130"/>
+        <item sd="0" x="131"/>
+        <item sd="0" x="132"/>
+        <item sd="0" x="133"/>
+        <item sd="0" x="134"/>
+        <item sd="0" x="135"/>
+        <item sd="0" x="136"/>
+        <item sd="0" x="137"/>
+        <item sd="0" x="138"/>
+        <item sd="0" x="139"/>
+        <item sd="0" x="140"/>
+        <item sd="0" x="141"/>
+        <item sd="0" x="142"/>
+        <item sd="0" x="143"/>
+        <item sd="0" x="144"/>
+        <item sd="0" x="145"/>
+        <item sd="0" x="146"/>
+        <item sd="0" x="147"/>
+        <item sd="0" x="148"/>
+        <item sd="0" x="149"/>
+        <item sd="0" x="150"/>
+        <item sd="0" x="151"/>
+        <item sd="0" x="152"/>
+        <item sd="0" x="153"/>
+        <item sd="0" x="154"/>
+        <item sd="0" x="155"/>
+        <item sd="0" x="156"/>
+        <item sd="0" x="157"/>
+        <item sd="0" x="158"/>
+        <item sd="0" x="159"/>
+        <item sd="0" x="160"/>
+        <item sd="0" x="161"/>
+        <item sd="0" x="162"/>
+        <item sd="0" x="163"/>
+        <item sd="0" x="164"/>
+        <item sd="0" x="165"/>
+        <item sd="0" x="166"/>
+        <item sd="0" x="167"/>
+        <item sd="0" x="168"/>
+        <item sd="0" x="169"/>
+        <item sd="0" x="170"/>
+        <item sd="0" x="171"/>
+        <item sd="0" x="172"/>
+        <item sd="0" x="173"/>
+        <item sd="0" x="174"/>
+        <item sd="0" x="175"/>
+        <item sd="0" x="176"/>
+        <item sd="0" x="177"/>
+        <item sd="0" x="178"/>
+        <item sd="0" x="179"/>
+        <item sd="0" x="180"/>
+        <item sd="0" x="181"/>
+        <item sd="0" x="182"/>
+        <item sd="0" x="183"/>
+        <item sd="0" x="184"/>
+        <item sd="0" x="185"/>
+        <item sd="0" x="186"/>
+        <item sd="0" x="187"/>
+        <item sd="0" x="188"/>
+        <item sd="0" x="189"/>
+        <item sd="0" x="190"/>
+        <item sd="0" x="191"/>
+        <item sd="0" x="192"/>
+        <item sd="0" x="193"/>
+        <item sd="0" x="194"/>
+        <item sd="0" x="195"/>
+        <item sd="0" x="196"/>
+        <item sd="0" x="197"/>
+        <item sd="0" x="198"/>
+        <item sd="0" x="199"/>
+        <item sd="0" x="200"/>
+        <item sd="0" x="201"/>
+        <item sd="0" x="202"/>
+        <item sd="0" x="203"/>
+        <item sd="0" x="204"/>
+        <item sd="0" x="205"/>
+        <item sd="0" x="206"/>
+        <item sd="0" x="207"/>
+        <item sd="0" x="208"/>
+        <item sd="0" x="209"/>
+        <item sd="0" x="210"/>
+        <item sd="0" x="211"/>
+        <item sd="0" x="212"/>
+        <item sd="0" x="213"/>
+        <item sd="0" x="214"/>
+        <item sd="0" x="215"/>
+        <item sd="0" x="216"/>
+        <item sd="0" x="217"/>
+        <item sd="0" x="218"/>
+        <item sd="0" x="219"/>
+        <item sd="0" x="220"/>
+        <item sd="0" x="221"/>
+        <item sd="0" x="222"/>
+        <item sd="0" x="223"/>
+        <item sd="0" x="224"/>
+        <item sd="0" x="225"/>
+        <item sd="0" x="226"/>
+        <item sd="0" x="227"/>
+        <item sd="0" x="228"/>
+        <item sd="0" x="229"/>
+        <item sd="0" x="230"/>
+        <item sd="0" x="231"/>
+        <item sd="0" x="232"/>
+        <item sd="0" x="233"/>
+        <item sd="0" x="234"/>
+        <item sd="0" x="235"/>
+        <item sd="0" x="236"/>
+        <item sd="0" x="237"/>
+        <item sd="0" x="238"/>
+        <item sd="0" x="239"/>
+        <item sd="0" x="240"/>
+        <item sd="0" x="241"/>
+        <item sd="0" x="242"/>
+        <item sd="0" x="243"/>
+        <item sd="0" x="244"/>
+        <item sd="0" x="245"/>
+        <item sd="0" x="246"/>
+        <item sd="0" x="247"/>
+        <item sd="0" x="248"/>
+        <item sd="0" x="249"/>
+        <item sd="0" x="250"/>
+        <item sd="0" x="251"/>
+        <item sd="0" x="252"/>
+        <item sd="0" x="253"/>
+        <item sd="0" x="254"/>
+        <item sd="0" x="255"/>
+        <item sd="0" x="256"/>
+        <item sd="0" x="257"/>
+        <item sd="0" x="258"/>
+        <item sd="0" x="259"/>
+        <item sd="0" x="260"/>
+        <item sd="0" x="261"/>
+        <item sd="0" x="262"/>
+        <item sd="0" x="263"/>
+        <item sd="0" x="264"/>
+        <item sd="0" x="265"/>
+        <item sd="0" x="266"/>
+        <item sd="0" x="267"/>
+        <item sd="0" x="268"/>
+        <item sd="0" x="269"/>
+        <item sd="0" x="270"/>
+        <item sd="0" x="271"/>
+        <item sd="0" x="272"/>
+        <item sd="0" x="273"/>
+        <item sd="0" x="274"/>
+        <item sd="0" x="275"/>
+        <item sd="0" x="276"/>
+        <item sd="0" x="277"/>
+        <item sd="0" x="278"/>
+        <item sd="0" x="279"/>
+        <item sd="0" x="280"/>
+        <item sd="0" x="281"/>
+        <item sd="0" x="282"/>
+        <item sd="0" x="283"/>
+        <item sd="0" x="284"/>
+        <item sd="0" x="285"/>
+        <item sd="0" x="286"/>
+        <item sd="0" x="287"/>
+        <item sd="0" x="288"/>
+        <item sd="0" x="289"/>
+        <item sd="0" x="290"/>
+        <item sd="0" x="291"/>
+        <item sd="0" x="292"/>
+        <item sd="0" x="293"/>
+        <item sd="0" x="294"/>
+        <item sd="0" x="295"/>
+        <item sd="0" x="296"/>
+        <item sd="0" x="297"/>
+        <item sd="0" x="298"/>
+        <item sd="0" x="299"/>
+        <item sd="0" x="300"/>
+        <item sd="0" x="301"/>
+        <item sd="0" x="302"/>
+        <item sd="0" x="303"/>
+        <item sd="0" x="304"/>
+        <item sd="0" x="305"/>
+        <item sd="0" x="306"/>
+        <item sd="0" x="307"/>
+        <item sd="0" x="308"/>
+        <item sd="0" x="309"/>
+        <item sd="0" x="310"/>
+        <item sd="0" x="311"/>
+        <item sd="0" x="312"/>
+        <item sd="0" x="313"/>
+        <item sd="0" x="314"/>
+        <item sd="0" x="315"/>
+        <item sd="0" x="316"/>
+        <item sd="0" x="317"/>
+        <item sd="0" x="318"/>
+        <item sd="0" x="319"/>
+        <item sd="0" x="320"/>
+        <item sd="0" x="321"/>
+        <item sd="0" x="322"/>
+        <item sd="0" x="323"/>
+        <item sd="0" x="324"/>
+        <item sd="0" x="325"/>
+        <item sd="0" x="326"/>
+        <item sd="0" x="327"/>
+        <item sd="0" x="328"/>
+        <item sd="0" x="329"/>
+        <item sd="0" x="330"/>
+        <item sd="0" x="331"/>
+        <item sd="0" x="332"/>
+        <item sd="0" x="333"/>
+        <item sd="0" x="334"/>
+        <item sd="0" x="335"/>
+        <item sd="0" x="336"/>
+        <item sd="0" x="337"/>
+        <item sd="0" x="338"/>
+        <item sd="0" x="339"/>
+        <item sd="0" x="340"/>
+        <item sd="0" x="341"/>
+        <item sd="0" x="342"/>
+        <item sd="0" x="343"/>
+        <item sd="0" x="344"/>
+        <item sd="0" x="345"/>
+        <item sd="0" x="346"/>
+        <item sd="0" x="347"/>
+        <item sd="0" x="348"/>
+        <item sd="0" x="349"/>
+        <item sd="0" x="350"/>
+        <item sd="0" x="351"/>
+        <item sd="0" x="352"/>
+        <item sd="0" x="353"/>
+        <item sd="0" x="354"/>
+        <item sd="0" x="355"/>
+        <item sd="0" x="356"/>
+        <item sd="0" x="357"/>
+        <item sd="0" x="358"/>
+        <item sd="0" x="359"/>
+        <item sd="0" x="360"/>
+        <item sd="0" x="361"/>
+        <item sd="0" x="362"/>
+        <item sd="0" x="363"/>
+        <item sd="0" x="364"/>
+        <item sd="0" x="365"/>
+        <item sd="0" x="366"/>
+        <item sd="0" x="367"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="14">
+        <item sd="0" x="0"/>
+        <item sd="0" x="1"/>
+        <item sd="0" x="2"/>
+        <item sd="0" x="3"/>
+        <item sd="0" x="4"/>
+        <item sd="0" x="5"/>
+        <item sd="0" x="6"/>
+        <item sd="0" x="7"/>
+        <item sd="0" x="8"/>
+        <item sd="0" x="9"/>
+        <item sd="0" x="10"/>
+        <item sd="0" x="11"/>
+        <item sd="0" x="12"/>
+        <item sd="0" x="13"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="2"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="6">
+    <chartFormat chart="2" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="2">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="3">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="1"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="4">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="2"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="5">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="6">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="2">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="4"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2EBA4ED6-0263-4163-B60D-94E9DAE81843}" name="Product Category Distribution" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="29">
+  <location ref="A39:B50" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0"/>
@@ -10492,8 +11122,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EEA1BD0D-A2BA-41BA-AC63-F069DCA73CCD}" name="Monthly Revenue Trends" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EEA1BD0D-A2BA-41BA-AC63-F069DCA73CCD}" name="Monthly Revenue Trends" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
   <location ref="A20:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -10990,8 +11620,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F701EDC3-81C2-4D13-8691-DB7E36575968}" name="Sales by Region" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F701EDC3-81C2-4D13-8691-DB7E36575968}" name="Sales by Region" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
   <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -11486,9 +12116,9 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EF61005-3DC2-4F04-A889-30AB3AB0D1A3}" name="Salesperson Performance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="13">
-  <location ref="A54:F63" firstHeaderRow="1" firstDataRow="4" firstDataCol="1"/>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EF61005-3DC2-4F04-A889-30AB3AB0D1A3}" name="Salesperson Performance Monthly" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+  <location ref="A64:F73" firstHeaderRow="1" firstDataRow="4" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0"/>
@@ -12155,9 +12785,9 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C975136F-C808-4BF6-9947-A39165D24CB0}" name="Products of the Month" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A44:G50" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C975136F-C808-4BF6-9947-A39165D24CB0}" name="Products of the Month" cacheId="1" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+  <location ref="A54:G60" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
     <pivotField numFmtId="14" showAll="0"/>
@@ -12731,563 +13361,6 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{77BF86ED-9B5C-443E-BA35-5E459117CD3F}" name="Top Performing Products" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
-  <location ref="A10:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="4"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="368">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-        <item sd="0" x="14"/>
-        <item sd="0" x="15"/>
-        <item sd="0" x="16"/>
-        <item sd="0" x="17"/>
-        <item sd="0" x="18"/>
-        <item sd="0" x="19"/>
-        <item sd="0" x="20"/>
-        <item sd="0" x="21"/>
-        <item sd="0" x="22"/>
-        <item sd="0" x="23"/>
-        <item sd="0" x="24"/>
-        <item sd="0" x="25"/>
-        <item sd="0" x="26"/>
-        <item sd="0" x="27"/>
-        <item sd="0" x="28"/>
-        <item sd="0" x="29"/>
-        <item sd="0" x="30"/>
-        <item sd="0" x="31"/>
-        <item sd="0" x="32"/>
-        <item sd="0" x="33"/>
-        <item sd="0" x="34"/>
-        <item sd="0" x="35"/>
-        <item sd="0" x="36"/>
-        <item sd="0" x="37"/>
-        <item sd="0" x="38"/>
-        <item sd="0" x="39"/>
-        <item sd="0" x="40"/>
-        <item sd="0" x="41"/>
-        <item sd="0" x="42"/>
-        <item sd="0" x="43"/>
-        <item sd="0" x="44"/>
-        <item sd="0" x="45"/>
-        <item sd="0" x="46"/>
-        <item sd="0" x="47"/>
-        <item sd="0" x="48"/>
-        <item sd="0" x="49"/>
-        <item sd="0" x="50"/>
-        <item sd="0" x="51"/>
-        <item sd="0" x="52"/>
-        <item sd="0" x="53"/>
-        <item sd="0" x="54"/>
-        <item sd="0" x="55"/>
-        <item sd="0" x="56"/>
-        <item sd="0" x="57"/>
-        <item sd="0" x="58"/>
-        <item sd="0" x="59"/>
-        <item sd="0" x="60"/>
-        <item sd="0" x="61"/>
-        <item sd="0" x="62"/>
-        <item sd="0" x="63"/>
-        <item sd="0" x="64"/>
-        <item sd="0" x="65"/>
-        <item sd="0" x="66"/>
-        <item sd="0" x="67"/>
-        <item sd="0" x="68"/>
-        <item sd="0" x="69"/>
-        <item sd="0" x="70"/>
-        <item sd="0" x="71"/>
-        <item sd="0" x="72"/>
-        <item sd="0" x="73"/>
-        <item sd="0" x="74"/>
-        <item sd="0" x="75"/>
-        <item sd="0" x="76"/>
-        <item sd="0" x="77"/>
-        <item sd="0" x="78"/>
-        <item sd="0" x="79"/>
-        <item sd="0" x="80"/>
-        <item sd="0" x="81"/>
-        <item sd="0" x="82"/>
-        <item sd="0" x="83"/>
-        <item sd="0" x="84"/>
-        <item sd="0" x="85"/>
-        <item sd="0" x="86"/>
-        <item sd="0" x="87"/>
-        <item sd="0" x="88"/>
-        <item sd="0" x="89"/>
-        <item sd="0" x="90"/>
-        <item sd="0" x="91"/>
-        <item sd="0" x="92"/>
-        <item sd="0" x="93"/>
-        <item sd="0" x="94"/>
-        <item sd="0" x="95"/>
-        <item sd="0" x="96"/>
-        <item sd="0" x="97"/>
-        <item sd="0" x="98"/>
-        <item sd="0" x="99"/>
-        <item sd="0" x="100"/>
-        <item sd="0" x="101"/>
-        <item sd="0" x="102"/>
-        <item sd="0" x="103"/>
-        <item sd="0" x="104"/>
-        <item sd="0" x="105"/>
-        <item sd="0" x="106"/>
-        <item sd="0" x="107"/>
-        <item sd="0" x="108"/>
-        <item sd="0" x="109"/>
-        <item sd="0" x="110"/>
-        <item sd="0" x="111"/>
-        <item sd="0" x="112"/>
-        <item sd="0" x="113"/>
-        <item sd="0" x="114"/>
-        <item sd="0" x="115"/>
-        <item sd="0" x="116"/>
-        <item sd="0" x="117"/>
-        <item sd="0" x="118"/>
-        <item sd="0" x="119"/>
-        <item sd="0" x="120"/>
-        <item sd="0" x="121"/>
-        <item sd="0" x="122"/>
-        <item sd="0" x="123"/>
-        <item sd="0" x="124"/>
-        <item sd="0" x="125"/>
-        <item sd="0" x="126"/>
-        <item sd="0" x="127"/>
-        <item sd="0" x="128"/>
-        <item sd="0" x="129"/>
-        <item sd="0" x="130"/>
-        <item sd="0" x="131"/>
-        <item sd="0" x="132"/>
-        <item sd="0" x="133"/>
-        <item sd="0" x="134"/>
-        <item sd="0" x="135"/>
-        <item sd="0" x="136"/>
-        <item sd="0" x="137"/>
-        <item sd="0" x="138"/>
-        <item sd="0" x="139"/>
-        <item sd="0" x="140"/>
-        <item sd="0" x="141"/>
-        <item sd="0" x="142"/>
-        <item sd="0" x="143"/>
-        <item sd="0" x="144"/>
-        <item sd="0" x="145"/>
-        <item sd="0" x="146"/>
-        <item sd="0" x="147"/>
-        <item sd="0" x="148"/>
-        <item sd="0" x="149"/>
-        <item sd="0" x="150"/>
-        <item sd="0" x="151"/>
-        <item sd="0" x="152"/>
-        <item sd="0" x="153"/>
-        <item sd="0" x="154"/>
-        <item sd="0" x="155"/>
-        <item sd="0" x="156"/>
-        <item sd="0" x="157"/>
-        <item sd="0" x="158"/>
-        <item sd="0" x="159"/>
-        <item sd="0" x="160"/>
-        <item sd="0" x="161"/>
-        <item sd="0" x="162"/>
-        <item sd="0" x="163"/>
-        <item sd="0" x="164"/>
-        <item sd="0" x="165"/>
-        <item sd="0" x="166"/>
-        <item sd="0" x="167"/>
-        <item sd="0" x="168"/>
-        <item sd="0" x="169"/>
-        <item sd="0" x="170"/>
-        <item sd="0" x="171"/>
-        <item sd="0" x="172"/>
-        <item sd="0" x="173"/>
-        <item sd="0" x="174"/>
-        <item sd="0" x="175"/>
-        <item sd="0" x="176"/>
-        <item sd="0" x="177"/>
-        <item sd="0" x="178"/>
-        <item sd="0" x="179"/>
-        <item sd="0" x="180"/>
-        <item sd="0" x="181"/>
-        <item sd="0" x="182"/>
-        <item sd="0" x="183"/>
-        <item sd="0" x="184"/>
-        <item sd="0" x="185"/>
-        <item sd="0" x="186"/>
-        <item sd="0" x="187"/>
-        <item sd="0" x="188"/>
-        <item sd="0" x="189"/>
-        <item sd="0" x="190"/>
-        <item sd="0" x="191"/>
-        <item sd="0" x="192"/>
-        <item sd="0" x="193"/>
-        <item sd="0" x="194"/>
-        <item sd="0" x="195"/>
-        <item sd="0" x="196"/>
-        <item sd="0" x="197"/>
-        <item sd="0" x="198"/>
-        <item sd="0" x="199"/>
-        <item sd="0" x="200"/>
-        <item sd="0" x="201"/>
-        <item sd="0" x="202"/>
-        <item sd="0" x="203"/>
-        <item sd="0" x="204"/>
-        <item sd="0" x="205"/>
-        <item sd="0" x="206"/>
-        <item sd="0" x="207"/>
-        <item sd="0" x="208"/>
-        <item sd="0" x="209"/>
-        <item sd="0" x="210"/>
-        <item sd="0" x="211"/>
-        <item sd="0" x="212"/>
-        <item sd="0" x="213"/>
-        <item sd="0" x="214"/>
-        <item sd="0" x="215"/>
-        <item sd="0" x="216"/>
-        <item sd="0" x="217"/>
-        <item sd="0" x="218"/>
-        <item sd="0" x="219"/>
-        <item sd="0" x="220"/>
-        <item sd="0" x="221"/>
-        <item sd="0" x="222"/>
-        <item sd="0" x="223"/>
-        <item sd="0" x="224"/>
-        <item sd="0" x="225"/>
-        <item sd="0" x="226"/>
-        <item sd="0" x="227"/>
-        <item sd="0" x="228"/>
-        <item sd="0" x="229"/>
-        <item sd="0" x="230"/>
-        <item sd="0" x="231"/>
-        <item sd="0" x="232"/>
-        <item sd="0" x="233"/>
-        <item sd="0" x="234"/>
-        <item sd="0" x="235"/>
-        <item sd="0" x="236"/>
-        <item sd="0" x="237"/>
-        <item sd="0" x="238"/>
-        <item sd="0" x="239"/>
-        <item sd="0" x="240"/>
-        <item sd="0" x="241"/>
-        <item sd="0" x="242"/>
-        <item sd="0" x="243"/>
-        <item sd="0" x="244"/>
-        <item sd="0" x="245"/>
-        <item sd="0" x="246"/>
-        <item sd="0" x="247"/>
-        <item sd="0" x="248"/>
-        <item sd="0" x="249"/>
-        <item sd="0" x="250"/>
-        <item sd="0" x="251"/>
-        <item sd="0" x="252"/>
-        <item sd="0" x="253"/>
-        <item sd="0" x="254"/>
-        <item sd="0" x="255"/>
-        <item sd="0" x="256"/>
-        <item sd="0" x="257"/>
-        <item sd="0" x="258"/>
-        <item sd="0" x="259"/>
-        <item sd="0" x="260"/>
-        <item sd="0" x="261"/>
-        <item sd="0" x="262"/>
-        <item sd="0" x="263"/>
-        <item sd="0" x="264"/>
-        <item sd="0" x="265"/>
-        <item sd="0" x="266"/>
-        <item sd="0" x="267"/>
-        <item sd="0" x="268"/>
-        <item sd="0" x="269"/>
-        <item sd="0" x="270"/>
-        <item sd="0" x="271"/>
-        <item sd="0" x="272"/>
-        <item sd="0" x="273"/>
-        <item sd="0" x="274"/>
-        <item sd="0" x="275"/>
-        <item sd="0" x="276"/>
-        <item sd="0" x="277"/>
-        <item sd="0" x="278"/>
-        <item sd="0" x="279"/>
-        <item sd="0" x="280"/>
-        <item sd="0" x="281"/>
-        <item sd="0" x="282"/>
-        <item sd="0" x="283"/>
-        <item sd="0" x="284"/>
-        <item sd="0" x="285"/>
-        <item sd="0" x="286"/>
-        <item sd="0" x="287"/>
-        <item sd="0" x="288"/>
-        <item sd="0" x="289"/>
-        <item sd="0" x="290"/>
-        <item sd="0" x="291"/>
-        <item sd="0" x="292"/>
-        <item sd="0" x="293"/>
-        <item sd="0" x="294"/>
-        <item sd="0" x="295"/>
-        <item sd="0" x="296"/>
-        <item sd="0" x="297"/>
-        <item sd="0" x="298"/>
-        <item sd="0" x="299"/>
-        <item sd="0" x="300"/>
-        <item sd="0" x="301"/>
-        <item sd="0" x="302"/>
-        <item sd="0" x="303"/>
-        <item sd="0" x="304"/>
-        <item sd="0" x="305"/>
-        <item sd="0" x="306"/>
-        <item sd="0" x="307"/>
-        <item sd="0" x="308"/>
-        <item sd="0" x="309"/>
-        <item sd="0" x="310"/>
-        <item sd="0" x="311"/>
-        <item sd="0" x="312"/>
-        <item sd="0" x="313"/>
-        <item sd="0" x="314"/>
-        <item sd="0" x="315"/>
-        <item sd="0" x="316"/>
-        <item sd="0" x="317"/>
-        <item sd="0" x="318"/>
-        <item sd="0" x="319"/>
-        <item sd="0" x="320"/>
-        <item sd="0" x="321"/>
-        <item sd="0" x="322"/>
-        <item sd="0" x="323"/>
-        <item sd="0" x="324"/>
-        <item sd="0" x="325"/>
-        <item sd="0" x="326"/>
-        <item sd="0" x="327"/>
-        <item sd="0" x="328"/>
-        <item sd="0" x="329"/>
-        <item sd="0" x="330"/>
-        <item sd="0" x="331"/>
-        <item sd="0" x="332"/>
-        <item sd="0" x="333"/>
-        <item sd="0" x="334"/>
-        <item sd="0" x="335"/>
-        <item sd="0" x="336"/>
-        <item sd="0" x="337"/>
-        <item sd="0" x="338"/>
-        <item sd="0" x="339"/>
-        <item sd="0" x="340"/>
-        <item sd="0" x="341"/>
-        <item sd="0" x="342"/>
-        <item sd="0" x="343"/>
-        <item sd="0" x="344"/>
-        <item sd="0" x="345"/>
-        <item sd="0" x="346"/>
-        <item sd="0" x="347"/>
-        <item sd="0" x="348"/>
-        <item sd="0" x="349"/>
-        <item sd="0" x="350"/>
-        <item sd="0" x="351"/>
-        <item sd="0" x="352"/>
-        <item sd="0" x="353"/>
-        <item sd="0" x="354"/>
-        <item sd="0" x="355"/>
-        <item sd="0" x="356"/>
-        <item sd="0" x="357"/>
-        <item sd="0" x="358"/>
-        <item sd="0" x="359"/>
-        <item sd="0" x="360"/>
-        <item sd="0" x="361"/>
-        <item sd="0" x="362"/>
-        <item sd="0" x="363"/>
-        <item sd="0" x="364"/>
-        <item sd="0" x="365"/>
-        <item sd="0" x="366"/>
-        <item sd="0" x="367"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="14">
-        <item sd="0" x="0"/>
-        <item sd="0" x="1"/>
-        <item sd="0" x="2"/>
-        <item sd="0" x="3"/>
-        <item sd="0" x="4"/>
-        <item sd="0" x="5"/>
-        <item sd="0" x="6"/>
-        <item sd="0" x="7"/>
-        <item sd="0" x="8"/>
-        <item sd="0" x="9"/>
-        <item sd="0" x="10"/>
-        <item sd="0" x="11"/>
-        <item sd="0" x="12"/>
-        <item sd="0" x="13"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="2"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="6">
-    <chartFormat chart="2" format="1" series="1">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="2">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="3">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="1"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="4">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="2"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="5">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="3"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-    <chartFormat chart="2" format="6">
-      <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="2">
-          <reference field="4294967294" count="1" selected="0">
-            <x v="0"/>
-          </reference>
-          <reference field="2" count="1" selected="0">
-            <x v="4"/>
-          </reference>
-        </references>
-      </pivotArea>
-    </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
 <file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
 <queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{4604BCA9-C72A-45E1-8FA9-C6178CEDFAF6}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
   <queryTableRefresh nextId="11">
@@ -13314,7 +13387,7 @@
     <pivotTable tabId="2" name="Sales by Region"/>
     <pivotTable tabId="2" name="Products of the Month"/>
     <pivotTable tabId="2" name="Top Performing Products"/>
-    <pivotTable tabId="2" name="Salesperson Performance"/>
+    <pivotTable tabId="2" name="Salesperson Performance Monthly"/>
     <pivotTable tabId="2" name="Product Category Distribution"/>
   </pivotTables>
   <data>
@@ -13336,7 +13409,7 @@
     <pivotTable tabId="2" name="Sales by Region"/>
     <pivotTable tabId="2" name="Products of the Month"/>
     <pivotTable tabId="2" name="Top Performing Products"/>
-    <pivotTable tabId="2" name="Salesperson Performance"/>
+    <pivotTable tabId="2" name="Salesperson Performance Monthly"/>
   </pivotTables>
   <data>
     <tabular pivotCacheId="755373820">
@@ -13382,7 +13455,7 @@
     <pivotTable tabId="2" name="Products of the Month"/>
     <pivotTable tabId="2" name="Sales by Region"/>
     <pivotTable tabId="2" name="Top Performing Products"/>
-    <pivotTable tabId="2" name="Salesperson Performance"/>
+    <pivotTable tabId="2" name="Salesperson Performance Monthly"/>
   </pivotTables>
   <data>
     <tabular pivotCacheId="755373820">
@@ -13716,7 +13789,7 @@
     <pivotTable tabId="2" name="Monthly Revenue Trends"/>
     <pivotTable tabId="2" name="Product Category Distribution"/>
     <pivotTable tabId="2" name="Products of the Month"/>
-    <pivotTable tabId="2" name="Salesperson Performance"/>
+    <pivotTable tabId="2" name="Salesperson Performance Monthly"/>
     <pivotTable tabId="2" name="Top Performing Products"/>
   </pivotTables>
   <state minimalRefreshVersion="6" lastRefreshVersion="6" pivotCacheId="755373820" filterType="unknown">
@@ -15326,13 +15399,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5FAD743A-8513-455B-83F4-D866E93A6E9D}">
-  <dimension ref="A1:G63"/>
+  <dimension ref="A1:G73"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="15" bestFit="1" customWidth="1"/>
     <col min="3" max="5" width="7.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="11.33203125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="16.5546875" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="9.21875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="10.88671875" bestFit="1" customWidth="1"/>
@@ -15535,211 +15609,138 @@
     </row>
     <row r="30" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A30" s="2" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="B30" s="7">
-        <v>58500</v>
+        <v>270000</v>
       </c>
     </row>
     <row r="31" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A31" s="3" t="s">
-        <v>21</v>
+      <c r="A31" s="2" t="s">
+        <v>13</v>
       </c>
       <c r="B31" s="7">
-        <v>58500</v>
+        <v>260500</v>
       </c>
     </row>
     <row r="32" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A32" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" s="7">
+        <v>204000</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A33" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="B33" s="7">
+        <v>148000</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A34" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="B34" s="7">
+        <v>21000</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A35" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B35" s="7">
+        <v>903500</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A39" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="B39" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A40" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B40" s="7">
+        <v>58500</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A41" s="3" t="s">
+        <v>21</v>
+      </c>
+      <c r="B41" s="7">
+        <v>58500</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A42" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="B32" s="7">
+      <c r="B42" s="7">
         <v>75000</v>
       </c>
     </row>
-    <row r="33" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A33" s="3" t="s">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A43" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="B33" s="7">
+      <c r="B43" s="7">
         <v>75000</v>
       </c>
     </row>
-    <row r="34" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A34" s="2" t="s">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A44" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B34" s="7">
+      <c r="B44" s="7">
         <v>180000</v>
       </c>
     </row>
-    <row r="35" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A35" s="3" t="s">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A45" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B35" s="7">
+      <c r="B45" s="7">
         <v>180000</v>
       </c>
     </row>
-    <row r="36" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A36" s="2" t="s">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A46" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B36" s="7">
+      <c r="B46" s="7">
         <v>440000</v>
       </c>
     </row>
-    <row r="37" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A37" s="3" t="s">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A47" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="B37" s="7">
+      <c r="B47" s="7">
         <v>440000</v>
       </c>
     </row>
-    <row r="38" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A38" s="2" t="s">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.3">
+      <c r="A48" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B38" s="7">
+      <c r="B48" s="7">
         <v>150000</v>
-      </c>
-    </row>
-    <row r="39" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A39" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="B39" s="7">
-        <v>150000</v>
-      </c>
-    </row>
-    <row r="40" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A40" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="B40" s="7">
-        <v>903500</v>
-      </c>
-    </row>
-    <row r="44" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A44" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B44" s="1" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="45" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A45" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="B45" t="s">
-        <v>24</v>
-      </c>
-      <c r="C45" t="s">
-        <v>20</v>
-      </c>
-      <c r="D45" t="s">
-        <v>10</v>
-      </c>
-      <c r="E45" t="s">
-        <v>14</v>
-      </c>
-      <c r="F45" t="s">
-        <v>17</v>
-      </c>
-      <c r="G45" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="46" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A46" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="B46" s="7"/>
-      <c r="C46" s="7">
-        <v>6000</v>
-      </c>
-      <c r="D46" s="7">
-        <v>36000</v>
-      </c>
-      <c r="E46" s="7">
-        <v>88000</v>
-      </c>
-      <c r="F46" s="7">
-        <v>30000</v>
-      </c>
-      <c r="G46" s="7">
-        <v>160000</v>
-      </c>
-    </row>
-    <row r="47" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A47" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="B47" s="7">
-        <v>22500</v>
-      </c>
-      <c r="C47" s="7">
-        <v>24000</v>
-      </c>
-      <c r="D47" s="7">
-        <v>36000</v>
-      </c>
-      <c r="E47" s="7">
-        <v>88000</v>
-      </c>
-      <c r="F47" s="7">
-        <v>30000</v>
-      </c>
-      <c r="G47" s="7">
-        <v>200500</v>
-      </c>
-    </row>
-    <row r="48" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A48" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="B48" s="7">
-        <v>22500</v>
-      </c>
-      <c r="C48" s="7">
-        <v>21000</v>
-      </c>
-      <c r="D48" s="7">
-        <v>60000</v>
-      </c>
-      <c r="E48" s="7">
-        <v>120000</v>
-      </c>
-      <c r="F48" s="7">
-        <v>48000</v>
-      </c>
-      <c r="G48" s="7">
-        <v>271500</v>
       </c>
     </row>
     <row r="49" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A49" s="2" t="s">
-        <v>33</v>
+      <c r="A49" s="3" t="s">
+        <v>11</v>
       </c>
       <c r="B49" s="7">
-        <v>13500</v>
-      </c>
-      <c r="C49" s="7">
-        <v>24000</v>
-      </c>
-      <c r="D49" s="7">
-        <v>48000</v>
-      </c>
-      <c r="E49" s="7">
-        <v>144000</v>
-      </c>
-      <c r="F49" s="7">
-        <v>42000</v>
-      </c>
-      <c r="G49" s="7">
-        <v>271500</v>
+        <v>150000</v>
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.3">
@@ -15747,21 +15748,6 @@
         <v>27</v>
       </c>
       <c r="B50" s="7">
-        <v>58500</v>
-      </c>
-      <c r="C50" s="7">
-        <v>75000</v>
-      </c>
-      <c r="D50" s="7">
-        <v>180000</v>
-      </c>
-      <c r="E50" s="7">
-        <v>440000</v>
-      </c>
-      <c r="F50" s="7">
-        <v>150000</v>
-      </c>
-      <c r="G50" s="7">
         <v>903500</v>
       </c>
     </row>
@@ -15774,140 +15760,284 @@
       </c>
     </row>
     <row r="55" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A55" s="1" t="s">
+        <v>26</v>
+      </c>
       <c r="B55" t="s">
+        <v>24</v>
+      </c>
+      <c r="C55" t="s">
+        <v>20</v>
+      </c>
+      <c r="D55" t="s">
+        <v>10</v>
+      </c>
+      <c r="E55" t="s">
+        <v>14</v>
+      </c>
+      <c r="F55" t="s">
+        <v>17</v>
+      </c>
+      <c r="G55" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="56" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A56" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C55" t="s">
-        <v>31</v>
-      </c>
-      <c r="D55" t="s">
-        <v>32</v>
-      </c>
-      <c r="E55" t="s">
-        <v>33</v>
-      </c>
-      <c r="F55" t="s">
-        <v>27</v>
+      <c r="B56" s="7"/>
+      <c r="C56" s="7">
+        <v>6000</v>
+      </c>
+      <c r="D56" s="7">
+        <v>36000</v>
+      </c>
+      <c r="E56" s="7">
+        <v>88000</v>
+      </c>
+      <c r="F56" s="7">
+        <v>30000</v>
+      </c>
+      <c r="G56" s="7">
+        <v>160000</v>
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A57" s="1" t="s">
-        <v>26</v>
+      <c r="A57" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="B57" s="7">
+        <v>22500</v>
+      </c>
+      <c r="C57" s="7">
+        <v>24000</v>
+      </c>
+      <c r="D57" s="7">
+        <v>36000</v>
+      </c>
+      <c r="E57" s="7">
+        <v>88000</v>
+      </c>
+      <c r="F57" s="7">
+        <v>30000</v>
+      </c>
+      <c r="G57" s="7">
+        <v>200500</v>
       </c>
     </row>
     <row r="58" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A58" s="2" t="s">
-        <v>19</v>
+        <v>32</v>
       </c>
       <c r="B58" s="7">
-        <v>66000</v>
+        <v>22500</v>
       </c>
       <c r="C58" s="7">
-        <v>36000</v>
+        <v>21000</v>
       </c>
       <c r="D58" s="7">
-        <v>96000</v>
+        <v>60000</v>
       </c>
       <c r="E58" s="7">
-        <v>72000</v>
+        <v>120000</v>
       </c>
       <c r="F58" s="7">
-        <v>270000</v>
+        <v>48000</v>
+      </c>
+      <c r="G58" s="7">
+        <v>271500</v>
       </c>
     </row>
     <row r="59" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A59" s="2" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="B59" s="7">
-        <v>30000</v>
+        <v>13500</v>
       </c>
       <c r="C59" s="7">
-        <v>81500</v>
+        <v>24000</v>
       </c>
       <c r="D59" s="7">
-        <v>55500</v>
+        <v>48000</v>
       </c>
       <c r="E59" s="7">
-        <v>93500</v>
+        <v>144000</v>
       </c>
       <c r="F59" s="7">
-        <v>260500</v>
+        <v>42000</v>
+      </c>
+      <c r="G59" s="7">
+        <v>271500</v>
       </c>
     </row>
     <row r="60" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A60" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="B60" s="7">
+        <v>58500</v>
+      </c>
+      <c r="C60" s="7">
+        <v>75000</v>
+      </c>
+      <c r="D60" s="7">
+        <v>180000</v>
+      </c>
+      <c r="E60" s="7">
+        <v>440000</v>
+      </c>
+      <c r="F60" s="7">
+        <v>150000</v>
+      </c>
+      <c r="G60" s="7">
+        <v>903500</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A64" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B65" t="s">
+        <v>30</v>
+      </c>
+      <c r="C65" t="s">
+        <v>31</v>
+      </c>
+      <c r="D65" t="s">
+        <v>32</v>
+      </c>
+      <c r="E65" t="s">
+        <v>33</v>
+      </c>
+      <c r="F65" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="1" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="B68" s="7">
+        <v>66000</v>
+      </c>
+      <c r="C68" s="7">
+        <v>36000</v>
+      </c>
+      <c r="D68" s="7">
+        <v>96000</v>
+      </c>
+      <c r="E68" s="7">
+        <v>72000</v>
+      </c>
+      <c r="F68" s="7">
+        <v>270000</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="B69" s="7">
+        <v>30000</v>
+      </c>
+      <c r="C69" s="7">
+        <v>81500</v>
+      </c>
+      <c r="D69" s="7">
+        <v>55500</v>
+      </c>
+      <c r="E69" s="7">
+        <v>93500</v>
+      </c>
+      <c r="F69" s="7">
+        <v>260500</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A70" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B60" s="7">
+      <c r="B70" s="7">
         <v>52000</v>
       </c>
-      <c r="C60" s="7">
+      <c r="C70" s="7">
         <v>21000</v>
       </c>
-      <c r="D60" s="7">
+      <c r="D70" s="7">
         <v>70000</v>
       </c>
-      <c r="E60" s="7">
+      <c r="E70" s="7">
         <v>61000</v>
       </c>
-      <c r="F60" s="7">
+      <c r="F70" s="7">
         <v>204000</v>
       </c>
     </row>
-    <row r="61" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A61" s="2" t="s">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="B61" s="7">
+      <c r="B71" s="7">
         <v>12000</v>
       </c>
-      <c r="C61" s="7">
+      <c r="C71" s="7">
         <v>53000</v>
       </c>
-      <c r="D61" s="7">
+      <c r="D71" s="7">
         <v>50000</v>
       </c>
-      <c r="E61" s="7">
+      <c r="E71" s="7">
         <v>33000</v>
       </c>
-      <c r="F61" s="7">
+      <c r="F71" s="7">
         <v>148000</v>
       </c>
     </row>
-    <row r="62" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A62" s="2" t="s">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="B62" s="7"/>
-      <c r="C62" s="7">
+      <c r="B72" s="7"/>
+      <c r="C72" s="7">
         <v>9000</v>
       </c>
-      <c r="D62" s="7"/>
-      <c r="E62" s="7">
+      <c r="D72" s="7"/>
+      <c r="E72" s="7">
         <v>12000</v>
       </c>
-      <c r="F62" s="7">
+      <c r="F72" s="7">
         <v>21000</v>
       </c>
     </row>
-    <row r="63" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A63" s="2" t="s">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="B63" s="7">
+      <c r="B73" s="7">
         <v>160000</v>
       </c>
-      <c r="C63" s="7">
+      <c r="C73" s="7">
         <v>200500</v>
       </c>
-      <c r="D63" s="7">
+      <c r="D73" s="7">
         <v>271500</v>
       </c>
-      <c r="E63" s="7">
+      <c r="E73" s="7">
         <v>271500</v>
       </c>
-      <c r="F63" s="7">
+      <c r="F73" s="7">
         <v>903500</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Commit changes to project
</commit_message>
<xml_diff>
--- a/Data Analysis Project/project/reports/Dashboard.xlsx
+++ b/Data Analysis Project/project/reports/Dashboard.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr hidePivotFieldList="1"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\sc_RushilJivan_2026\Data Analysis Project\project\reports\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F8723CD-5E54-4231-A5E4-956AFAE8B286}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5640A4EC-8CB7-47D5-B628-C7126203F311}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
   <definedNames>
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">'clean_sales'!$A$1:$J$49</definedName>
     <definedName name="NativeTimeline_month">#N/A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="2">Dashboard!$A$1:$AK$49</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="2">Dashboard!$A$1:$AL$55</definedName>
     <definedName name="Slicer_category">#N/A</definedName>
     <definedName name="Slicer_product">#N/A</definedName>
     <definedName name="Slicer_region">#N/A</definedName>
@@ -661,7 +661,11 @@
         <c:crossBetween val="between"/>
       </c:valAx>
       <c:spPr>
-        <a:noFill/>
+        <a:solidFill>
+          <a:schemeClr val="bg1">
+            <a:lumMod val="95000"/>
+          </a:schemeClr>
+        </a:solidFill>
         <a:ln>
           <a:noFill/>
         </a:ln>
@@ -1286,6 +1290,43 @@
         <c:marker>
           <c:symbol val="none"/>
         </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="6"/>
@@ -1301,6 +1342,43 @@
         <c:marker>
           <c:symbol val="none"/>
         </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="7"/>
@@ -1316,6 +1394,43 @@
         <c:marker>
           <c:symbol val="none"/>
         </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="8"/>
@@ -1331,6 +1446,43 @@
         <c:marker>
           <c:symbol val="none"/>
         </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="9"/>
@@ -1346,6 +1498,43 @@
         <c:marker>
           <c:symbol val="none"/>
         </c:marker>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
       </c:pivotFmt>
       <c:pivotFmt>
         <c:idx val="10"/>
@@ -1403,6 +1592,120 @@
           </c:extLst>
         </c:dLbl>
       </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="11"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent5">
+              <a:tint val="54000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="-1.1980309841942451E-2"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
+      <c:pivotFmt>
+        <c:idx val="12"/>
+        <c:spPr>
+          <a:solidFill>
+            <a:schemeClr val="accent5">
+              <a:tint val="54000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+          <a:effectLst/>
+        </c:spPr>
+        <c:dLbl>
+          <c:idx val="0"/>
+          <c:layout>
+            <c:manualLayout>
+              <c:x val="-1.1980309841942451E-2"/>
+              <c:y val="0"/>
+            </c:manualLayout>
+          </c:layout>
+          <c:spPr>
+            <a:noFill/>
+            <a:ln>
+              <a:noFill/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:txPr>
+            <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+            <a:lstStyle/>
+            <a:p>
+              <a:pPr>
+                <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                  <a:solidFill>
+                    <a:sysClr val="windowText" lastClr="000000"/>
+                  </a:solidFill>
+                  <a:latin typeface="+mn-lt"/>
+                  <a:ea typeface="+mn-ea"/>
+                  <a:cs typeface="+mn-cs"/>
+                </a:defRPr>
+              </a:pPr>
+              <a:endParaRPr lang="en-US"/>
+            </a:p>
+          </c:txPr>
+          <c:dLblPos val="outEnd"/>
+          <c:showLegendKey val="0"/>
+          <c:showVal val="1"/>
+          <c:showCatName val="0"/>
+          <c:showSerName val="0"/>
+          <c:showPercent val="0"/>
+          <c:showBubbleSize val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+          </c:extLst>
+        </c:dLbl>
+      </c:pivotFmt>
     </c:pivotFmts>
     <c:plotArea>
       <c:layout/>
@@ -1436,6 +1739,145 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dPt>
+            <c:idx val="1"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:tint val="54000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000001-2DB3-4E06-B608-BA76B17E4A92}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dPt>
+            <c:idx val="2"/>
+            <c:invertIfNegative val="0"/>
+            <c:bubble3D val="0"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5">
+                  <a:tint val="54000"/>
+                </a:schemeClr>
+              </a:solidFill>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:extLst>
+              <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                <c16:uniqueId val="{00000000-2DB3-4E06-B608-BA76B17E4A92}"/>
+              </c:ext>
+            </c:extLst>
+          </c:dPt>
+          <c:dLbls>
+            <c:dLbl>
+              <c:idx val="1"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.1980309841942451E-2"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000001-2DB3-4E06-B608-BA76B17E4A92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:dLbl>
+              <c:idx val="2"/>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="-1.1980309841942451E-2"/>
+                  <c:y val="0"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:dLblPos val="outEnd"/>
+              <c:showLegendKey val="0"/>
+              <c:showVal val="1"/>
+              <c:showCatName val="0"/>
+              <c:showSerName val="0"/>
+              <c:showPercent val="0"/>
+              <c:showBubbleSize val="0"/>
+              <c:extLst>
+                <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
+                <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+                  <c16:uniqueId val="{00000000-2DB3-4E06-B608-BA76B17E4A92}"/>
+                </c:ext>
+              </c:extLst>
+            </c:dLbl>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Pivot_Tables!$A$56:$A$60</c:f>
@@ -1506,6 +1948,59 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Pivot_Tables!$A$56:$A$60</c:f>
@@ -1549,7 +2044,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000013-562A-4153-A0B4-C37AEFF8267D}"/>
+              <c16:uniqueId val="{00000014-5AB3-442E-9EA0-5AFB8455F704}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1577,6 +2072,59 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Pivot_Tables!$A$56:$A$60</c:f>
@@ -1620,7 +2168,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000001-B0B2-4298-825C-1ED712429386}"/>
+              <c16:uniqueId val="{00000005-A775-494E-9C67-68C7950BD0FE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1650,6 +2198,59 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Pivot_Tables!$A$56:$A$60</c:f>
@@ -1693,7 +2294,7 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-B0B2-4298-825C-1ED712429386}"/>
+              <c16:uniqueId val="{00000006-A775-494E-9C67-68C7950BD0FE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -1723,6 +2324,59 @@
             <a:effectLst/>
           </c:spPr>
           <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln>
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:txPr>
+              <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr sz="1050" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                    <a:solidFill>
+                      <a:sysClr val="windowText" lastClr="000000"/>
+                    </a:solidFill>
+                    <a:latin typeface="+mn-lt"/>
+                    <a:ea typeface="+mn-ea"/>
+                    <a:cs typeface="+mn-cs"/>
+                  </a:defRPr>
+                </a:pPr>
+                <a:endParaRPr lang="en-US"/>
+              </a:p>
+            </c:txPr>
+            <c:dLblPos val="outEnd"/>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="1"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:showBubbleSize val="0"/>
+            <c:showLeaderLines val="0"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+                <c15:leaderLines>
+                  <c:spPr>
+                    <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+                      <a:solidFill>
+                        <a:schemeClr val="tx1">
+                          <a:lumMod val="35000"/>
+                          <a:lumOff val="65000"/>
+                        </a:schemeClr>
+                      </a:solidFill>
+                      <a:round/>
+                    </a:ln>
+                    <a:effectLst/>
+                  </c:spPr>
+                </c15:leaderLines>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
           <c:cat>
             <c:strRef>
               <c:f>Pivot_Tables!$A$56:$A$60</c:f>
@@ -1766,14 +2420,14 @@
           </c:val>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000003-B0B2-4298-825C-1ED712429386}"/>
+              <c16:uniqueId val="{00000007-A775-494E-9C67-68C7950BD0FE}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:dLbls>
-          <c:dLblPos val="ctr"/>
+          <c:dLblPos val="outEnd"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
@@ -1815,7 +2469,7 @@
             <a:pPr>
               <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1"/>
+                  <a:sysClr val="windowText" lastClr="000000"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -1871,7 +2525,7 @@
             <a:pPr>
               <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                 <a:solidFill>
-                  <a:schemeClr val="tx1"/>
+                  <a:sysClr val="windowText" lastClr="000000"/>
                 </a:solidFill>
                 <a:latin typeface="+mn-lt"/>
                 <a:ea typeface="+mn-ea"/>
@@ -1910,7 +2564,7 @@
           <a:pPr>
             <a:defRPr sz="1100" b="1" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
               <a:solidFill>
-                <a:schemeClr val="tx1"/>
+                <a:sysClr val="windowText" lastClr="000000"/>
               </a:solidFill>
               <a:latin typeface="+mn-lt"/>
               <a:ea typeface="+mn-ea"/>
@@ -1954,7 +2608,11 @@
     <a:lstStyle/>
     <a:p>
       <a:pPr>
-        <a:defRPr/>
+        <a:defRPr sz="1050">
+          <a:solidFill>
+            <a:sysClr val="windowText" lastClr="000000"/>
+          </a:solidFill>
+        </a:defRPr>
       </a:pPr>
       <a:endParaRPr lang="en-US"/>
     </a:p>
@@ -3706,7 +4364,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{0000000F-AAEE-4E8A-BEC2-1BF2200785A1}"/>
+              <c16:uniqueId val="{0000000F-9245-4E60-8266-BB18CB3F7EF9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4070,7 +4728,7 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000010-AAEE-4E8A-BEC2-1BF2200785A1}"/>
+              <c16:uniqueId val="{00000010-9245-4E60-8266-BB18CB3F7EF9}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -4386,6 +5044,7 @@
         </c:marker>
         <c:dLbl>
           <c:idx val="0"/>
+          <c:numFmt formatCode="0%" sourceLinked="0"/>
           <c:spPr>
             <a:noFill/>
             <a:ln>
@@ -4618,6 +5277,7 @@
             </c:extLst>
           </c:dPt>
           <c:dLbls>
+            <c:numFmt formatCode="0%" sourceLinked="0"/>
             <c:spPr>
               <a:noFill/>
               <a:ln>
@@ -4651,21 +5311,7 @@
             <c:showSerName val="0"/>
             <c:showPercent val="1"/>
             <c:showBubbleSize val="0"/>
-            <c:showLeaderLines val="1"/>
-            <c:leaderLines>
-              <c:spPr>
-                <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
-                  <a:solidFill>
-                    <a:schemeClr val="tx1">
-                      <a:lumMod val="35000"/>
-                      <a:lumOff val="65000"/>
-                    </a:schemeClr>
-                  </a:solidFill>
-                  <a:round/>
-                </a:ln>
-                <a:effectLst/>
-              </c:spPr>
-            </c:leaderLines>
+            <c:showLeaderLines val="0"/>
             <c:extLst>
               <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}"/>
             </c:extLst>
@@ -4743,13 +5389,14 @@
           </c:extLst>
         </c:ser>
         <c:dLbls>
+          <c:dLblPos val="bestFit"/>
           <c:showLegendKey val="0"/>
-          <c:showVal val="0"/>
+          <c:showVal val="1"/>
           <c:showCatName val="0"/>
           <c:showSerName val="0"/>
           <c:showPercent val="0"/>
           <c:showBubbleSize val="0"/>
-          <c:showLeaderLines val="1"/>
+          <c:showLeaderLines val="0"/>
         </c:dLbls>
         <c:firstSliceAng val="0"/>
       </c:pieChart>
@@ -7502,101 +8149,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>22413</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>22412</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>578290</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>184889</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>14941</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>22412</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="5" name="Rectangle 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FF21DA0-0DFC-D5F0-D186-A41CE0DD4B2B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="22413" y="22412"/>
-          <a:ext cx="22658293" cy="537882"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="75000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-ZA" sz="2800" b="1" u="none">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>Sales</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-ZA" sz="2800" b="1" u="none" baseline="0">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t> Analysis Dashboard</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-ZA" sz="2800" b="1" u="none">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>28756</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>28756</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>576831</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>1</xdr:rowOff>
+      <xdr:rowOff>159728</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -7611,8 +8173,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="28756" y="556294"/>
-          <a:ext cx="5510398" cy="498784"/>
+          <a:off x="7824479" y="745606"/>
+          <a:ext cx="5433182" cy="535556"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7673,16 +8235,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>23671</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>561087</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>34728</xdr:rowOff>
+      <xdr:rowOff>164585</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>54709</xdr:colOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>591630</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>5310</xdr:rowOff>
+      <xdr:rowOff>138761</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -7697,8 +8259,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="6067119" y="586521"/>
-          <a:ext cx="5470142" cy="522375"/>
+          <a:off x="13845766" y="725302"/>
+          <a:ext cx="5465185" cy="534893"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7746,16 +8308,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>580476</xdr:colOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>579237</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>21845</xdr:rowOff>
+      <xdr:rowOff>164840</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>28</xdr:col>
-      <xdr:colOff>609599</xdr:colOff>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>4014</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>11724</xdr:rowOff>
+      <xdr:rowOff>158313</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -7770,8 +8332,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="12162876" y="584553"/>
-          <a:ext cx="5515523" cy="552586"/>
+          <a:off x="19902407" y="725557"/>
+          <a:ext cx="5463267" cy="554190"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -7830,73 +8392,161 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>350520</xdr:colOff>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>8036</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>3</xdr:col>
-      <xdr:colOff>388620</xdr:colOff>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>564</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>3224</xdr:rowOff>
+      <xdr:rowOff>0</xdr:rowOff>
     </xdr:to>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="13" name="Picture 12">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="11" name="Group 10">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6DE4EE44-2882-ECBC-7530-F9652EE7C7B3}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B2127BD8-DC66-5E78-9107-EA3050AA9663}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" r:link="rId2">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
         <a:xfrm>
-          <a:off x="350520" y="30480"/>
-          <a:ext cx="1891614" cy="519293"/>
+          <a:off x="3031846" y="0"/>
+          <a:ext cx="22368718" cy="544286"/>
+          <a:chOff x="22413" y="22412"/>
+          <a:chExt cx="22334943" cy="560717"/>
         </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="5" name="Rectangle 4">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0FF21DA0-0DFC-D5F0-D186-A41CE0DD4B2B}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="22413" y="22412"/>
+            <a:ext cx="22334943" cy="560717"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="accent5"/>
+          </a:solidFill>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-ZA" sz="2800" b="1" u="none">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Sales</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-ZA" sz="2800" b="1" u="none" baseline="0">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t> Analysis Dashboard</a:t>
+            </a:r>
+            <a:endParaRPr lang="en-ZA" sz="2800" b="1" u="none">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="13" name="Picture 12">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{6DE4EE44-2882-ECBC-7530-F9652EE7C7B3}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" r:link="rId2">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:srcRect/>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr bwMode="auto">
+          <a:xfrm>
+            <a:off x="350520" y="30480"/>
+            <a:ext cx="1849647" cy="533461"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
           <a:noFill/>
-        </a:ln>
-      </xdr:spPr>
-    </xdr:pic>
+          <a:ln>
+            <a:noFill/>
+          </a:ln>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>576829</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>20946</xdr:rowOff>
+      <xdr:rowOff>177079</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:col>21</xdr:col>
+      <xdr:colOff>576830</xdr:colOff>
       <xdr:row>23</xdr:row>
-      <xdr:rowOff>29307</xdr:rowOff>
+      <xdr:rowOff>185440</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7923,16 +8573,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>10</xdr:col>
-      <xdr:colOff>20067</xdr:colOff>
+      <xdr:col>22</xdr:col>
+      <xdr:colOff>550362</xdr:colOff>
       <xdr:row>6</xdr:row>
-      <xdr:rowOff>26399</xdr:rowOff>
+      <xdr:rowOff>152728</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>35442</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>159488</xdr:rowOff>
+      <xdr:col>31</xdr:col>
+      <xdr:colOff>590949</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>95317</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -7957,329 +8607,18 @@
     </xdr:graphicFrame>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>605780</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>36129</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>589471</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>109800</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>35034</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>32403</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="17" name="category">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE139141-239D-A45A-08DF-E3E485C7CB1C}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="category"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="18131780" y="2059370"/>
-              <a:ext cx="4264013" cy="915930"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-ZA" sz="1100"/>
-                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
-If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>609996</xdr:colOff>
-      <xdr:row>16</xdr:row>
-      <xdr:rowOff>41615</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>35034</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>37888</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="18" name="region">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7080A43D-BE88-E7D7-3C49-21FAB330A633}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="region"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="18135996" y="2984512"/>
-              <a:ext cx="4259797" cy="915928"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-ZA" sz="1100"/>
-                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
-If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>605806</xdr:colOff>
-      <xdr:row>21</xdr:row>
-      <xdr:rowOff>48966</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>35033</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>46596</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="19" name="salesperson">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27F4B1E2-B87B-0BAC-D8FA-544DBABD133B}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="salesperson"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="18131806" y="3911518"/>
-              <a:ext cx="4263986" cy="917285"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-ZA" sz="1100"/>
-                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
-If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
-    <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>606206</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>21511</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>17517</xdr:colOff>
-      <xdr:row>11</xdr:row>
-      <xdr:rowOff>17784</xdr:rowOff>
-    </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer">
-      <mc:Choice Requires="tsle">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="22" name="month">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5ACBCBBD-9EBB-4693-821C-A458E5FEA729}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2012/timeslicer">
-              <tsle:timeslicer name="month"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="18132206" y="1125097"/>
-              <a:ext cx="4246070" cy="915928"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
-              <a:solidFill>
-                <a:prstClr val="green"/>
-              </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-ZA" sz="1100"/>
-                <a:t>Timeline: Works in Excel 2013 or higher. Do not move or resize.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>153712</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>600808</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>152078</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>586432</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>169271</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8306,16 +8645,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>34615</xdr:colOff>
+      <xdr:col>13</xdr:col>
+      <xdr:colOff>20237</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>10850</xdr:rowOff>
+      <xdr:rowOff>157438</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>13</xdr:col>
-      <xdr:colOff>607840</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>158988</xdr:rowOff>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>592968</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>115076</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -8330,8 +8669,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="34615" y="4582850"/>
-          <a:ext cx="8498025" cy="513898"/>
+          <a:off x="7870275" y="4830080"/>
+          <a:ext cx="8422768" cy="518354"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8377,169 +8716,425 @@
     </xdr:sp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>608297</xdr:colOff>
-      <xdr:row>26</xdr:row>
-      <xdr:rowOff>73745</xdr:rowOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>589472</xdr:colOff>
+      <xdr:row>25</xdr:row>
+      <xdr:rowOff>159728</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>35034</xdr:colOff>
-      <xdr:row>31</xdr:row>
-      <xdr:rowOff>70018</xdr:rowOff>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>19221</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>146587</xdr:rowOff>
     </xdr:to>
-    <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-      <mc:Choice Requires="a14">
-        <xdr:graphicFrame macro="">
-          <xdr:nvGraphicFramePr>
-            <xdr:cNvPr id="27" name="product">
-              <a:extLst>
-                <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                  <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B75EB513-CF99-3882-D2F1-55E02D991CB7}"/>
-                </a:ext>
-              </a:extLst>
-            </xdr:cNvPr>
-            <xdr:cNvGraphicFramePr/>
-          </xdr:nvGraphicFramePr>
-          <xdr:xfrm>
-            <a:off x="0" y="0"/>
-            <a:ext cx="0" cy="0"/>
-          </xdr:xfrm>
-          <a:graphic>
-            <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
-              <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="product"/>
-            </a:graphicData>
-          </a:graphic>
-        </xdr:graphicFrame>
-      </mc:Choice>
-      <mc:Fallback xmlns="">
-        <xdr:sp macro="" textlink="">
-          <xdr:nvSpPr>
-            <xdr:cNvPr id="0" name=""/>
-            <xdr:cNvSpPr>
-              <a:spLocks noTextEdit="1"/>
-            </xdr:cNvSpPr>
-          </xdr:nvSpPr>
-          <xdr:spPr>
-            <a:xfrm>
-              <a:off x="18286697" y="4696545"/>
-              <a:ext cx="4303537" cy="885273"/>
-            </a:xfrm>
-            <a:prstGeom prst="rect">
-              <a:avLst/>
-            </a:prstGeom>
-            <a:solidFill>
-              <a:prstClr val="white"/>
-            </a:solidFill>
-            <a:ln w="1">
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="16" name="Group 15">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{0238F9C9-7FE9-CCB9-0373-EB319F40BE49}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="3008520" y="4695442"/>
+          <a:ext cx="4267844" cy="4885431"/>
+          <a:chOff x="0" y="4529005"/>
+          <a:chExt cx="4300799" cy="4849806"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+          <xdr:graphicFrame macro="">
+            <xdr:nvGraphicFramePr>
+              <xdr:cNvPr id="17" name="category">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CE139141-239D-A45A-08DF-E3E485C7CB1C}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
+              <xdr:cNvGraphicFramePr/>
+            </xdr:nvGraphicFramePr>
+            <xdr:xfrm>
+              <a:off x="0" y="5902754"/>
+              <a:ext cx="4300799" cy="855984"/>
+            </xdr:xfrm>
+            <a:graphic>
+              <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+                <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="category"/>
+              </a:graphicData>
+            </a:graphic>
+          </xdr:graphicFrame>
+        </mc:Choice>
+        <mc:Fallback>
+          <xdr:sp macro="" textlink="">
+            <xdr:nvSpPr>
+              <xdr:cNvPr id="0" name=""/>
+              <xdr:cNvSpPr>
+                <a:spLocks noTextEdit="1"/>
+              </xdr:cNvSpPr>
+            </xdr:nvSpPr>
+            <xdr:spPr>
+              <a:xfrm>
+                <a:off x="3008520" y="6079282"/>
+                <a:ext cx="4267844" cy="862272"/>
+              </a:xfrm>
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
               <a:solidFill>
-                <a:prstClr val="green"/>
+                <a:prstClr val="white"/>
               </a:solidFill>
-            </a:ln>
-          </xdr:spPr>
-          <xdr:txBody>
-            <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
-            <a:lstStyle/>
-            <a:p>
-              <a:r>
-                <a:rPr lang="en-ZA" sz="1100"/>
-                <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+              <a:ln w="1">
+                <a:solidFill>
+                  <a:prstClr val="green"/>
+                </a:solidFill>
+              </a:ln>
+            </xdr:spPr>
+            <xdr:txBody>
+              <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:rPr lang="en-ZA" sz="1100"/>
+                  <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
 If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
-              </a:r>
-            </a:p>
-          </xdr:txBody>
-        </xdr:sp>
-      </mc:Fallback>
-    </mc:AlternateContent>
+                </a:r>
+              </a:p>
+            </xdr:txBody>
+          </xdr:sp>
+        </mc:Fallback>
+      </mc:AlternateContent>
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+          <xdr:graphicFrame macro="">
+            <xdr:nvGraphicFramePr>
+              <xdr:cNvPr id="18" name="region">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{7080A43D-BE88-E7D7-3C49-21FAB330A633}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
+              <xdr:cNvGraphicFramePr/>
+            </xdr:nvGraphicFramePr>
+            <xdr:xfrm>
+              <a:off x="4269" y="6767228"/>
+              <a:ext cx="4296530" cy="855982"/>
+            </xdr:xfrm>
+            <a:graphic>
+              <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+                <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="region"/>
+              </a:graphicData>
+            </a:graphic>
+          </xdr:graphicFrame>
+        </mc:Choice>
+        <mc:Fallback>
+          <xdr:sp macro="" textlink="">
+            <xdr:nvSpPr>
+              <xdr:cNvPr id="0" name=""/>
+              <xdr:cNvSpPr>
+                <a:spLocks noTextEdit="1"/>
+              </xdr:cNvSpPr>
+            </xdr:nvSpPr>
+            <xdr:spPr>
+              <a:xfrm>
+                <a:off x="3012756" y="6950106"/>
+                <a:ext cx="4263608" cy="862270"/>
+              </a:xfrm>
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:solidFill>
+                <a:prstClr val="white"/>
+              </a:solidFill>
+              <a:ln w="1">
+                <a:solidFill>
+                  <a:prstClr val="green"/>
+                </a:solidFill>
+              </a:ln>
+            </xdr:spPr>
+            <xdr:txBody>
+              <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:rPr lang="en-ZA" sz="1100"/>
+                  <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+                </a:r>
+              </a:p>
+            </xdr:txBody>
+          </xdr:sp>
+        </mc:Fallback>
+      </mc:AlternateContent>
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+          <xdr:graphicFrame macro="">
+            <xdr:nvGraphicFramePr>
+              <xdr:cNvPr id="19" name="salesperson">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{27F4B1E2-B87B-0BAC-D8FA-544DBABD133B}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
+              <xdr:cNvGraphicFramePr/>
+            </xdr:nvGraphicFramePr>
+            <xdr:xfrm>
+              <a:off x="26" y="7633419"/>
+              <a:ext cx="4300772" cy="857232"/>
+            </xdr:xfrm>
+            <a:graphic>
+              <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+                <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="salesperson"/>
+              </a:graphicData>
+            </a:graphic>
+          </xdr:graphicFrame>
+        </mc:Choice>
+        <mc:Fallback>
+          <xdr:sp macro="" textlink="">
+            <xdr:nvSpPr>
+              <xdr:cNvPr id="0" name=""/>
+              <xdr:cNvSpPr>
+                <a:spLocks noTextEdit="1"/>
+              </xdr:cNvSpPr>
+            </xdr:nvSpPr>
+            <xdr:spPr>
+              <a:xfrm>
+                <a:off x="3008546" y="7822660"/>
+                <a:ext cx="4267817" cy="863529"/>
+              </a:xfrm>
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:solidFill>
+                <a:prstClr val="white"/>
+              </a:solidFill>
+              <a:ln w="1">
+                <a:solidFill>
+                  <a:prstClr val="green"/>
+                </a:solidFill>
+              </a:ln>
+            </xdr:spPr>
+            <xdr:txBody>
+              <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:rPr lang="en-ZA" sz="1100"/>
+                  <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+                </a:r>
+              </a:p>
+            </xdr:txBody>
+          </xdr:sp>
+        </mc:Fallback>
+      </mc:AlternateContent>
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" Requires="tsle">
+          <xdr:graphicFrame macro="">
+            <xdr:nvGraphicFramePr>
+              <xdr:cNvPr id="22" name="month">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5ACBCBBD-9EBB-4693-821C-A458E5FEA729}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
+              <xdr:cNvGraphicFramePr/>
+            </xdr:nvGraphicFramePr>
+            <xdr:xfrm>
+              <a:off x="432" y="5029867"/>
+              <a:ext cx="4282629" cy="855983"/>
+            </xdr:xfrm>
+            <a:graphic>
+              <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2012/timeslicer">
+                <tsle:timeslicer xmlns:tsle="http://schemas.microsoft.com/office/drawing/2012/timeslicer" name="month"/>
+              </a:graphicData>
+            </a:graphic>
+          </xdr:graphicFrame>
+        </mc:Choice>
+        <mc:Fallback>
+          <xdr:sp macro="" textlink="">
+            <xdr:nvSpPr>
+              <xdr:cNvPr id="0" name=""/>
+              <xdr:cNvSpPr>
+                <a:spLocks noTextEdit="1"/>
+              </xdr:cNvSpPr>
+            </xdr:nvSpPr>
+            <xdr:spPr>
+              <a:xfrm>
+                <a:off x="3008949" y="5199983"/>
+                <a:ext cx="4249813" cy="862271"/>
+              </a:xfrm>
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:solidFill>
+                <a:prstClr val="white"/>
+              </a:solidFill>
+              <a:ln w="1">
+                <a:solidFill>
+                  <a:prstClr val="green"/>
+                </a:solidFill>
+              </a:ln>
+            </xdr:spPr>
+            <xdr:txBody>
+              <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:rPr lang="en-ZA" sz="1100"/>
+                  <a:t>Timeline: Works in Excel 2013 or higher. Do not move or resize.</a:t>
+                </a:r>
+              </a:p>
+            </xdr:txBody>
+          </xdr:sp>
+        </mc:Fallback>
+      </mc:AlternateContent>
+      <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+        <mc:Choice xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" Requires="a14">
+          <xdr:graphicFrame macro="">
+            <xdr:nvGraphicFramePr>
+              <xdr:cNvPr id="27" name="product">
+                <a:extLst>
+                  <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                    <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B75EB513-CF99-3882-D2F1-55E02D991CB7}"/>
+                  </a:ext>
+                </a:extLst>
+              </xdr:cNvPr>
+              <xdr:cNvGraphicFramePr/>
+            </xdr:nvGraphicFramePr>
+            <xdr:xfrm>
+              <a:off x="2549" y="8522828"/>
+              <a:ext cx="4298250" cy="855983"/>
+            </xdr:xfrm>
+            <a:graphic>
+              <a:graphicData uri="http://schemas.microsoft.com/office/drawing/2010/slicer">
+                <sle:slicer xmlns:sle="http://schemas.microsoft.com/office/drawing/2010/slicer" name="product"/>
+              </a:graphicData>
+            </a:graphic>
+          </xdr:graphicFrame>
+        </mc:Choice>
+        <mc:Fallback>
+          <xdr:sp macro="" textlink="">
+            <xdr:nvSpPr>
+              <xdr:cNvPr id="0" name=""/>
+              <xdr:cNvSpPr>
+                <a:spLocks noTextEdit="1"/>
+              </xdr:cNvSpPr>
+            </xdr:nvSpPr>
+            <xdr:spPr>
+              <a:xfrm>
+                <a:off x="3011049" y="8718602"/>
+                <a:ext cx="4265315" cy="862271"/>
+              </a:xfrm>
+              <a:prstGeom prst="rect">
+                <a:avLst/>
+              </a:prstGeom>
+              <a:solidFill>
+                <a:prstClr val="white"/>
+              </a:solidFill>
+              <a:ln w="1">
+                <a:solidFill>
+                  <a:prstClr val="green"/>
+                </a:solidFill>
+              </a:ln>
+            </xdr:spPr>
+            <xdr:txBody>
+              <a:bodyPr vertOverflow="clip" horzOverflow="clip"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:r>
+                  <a:rPr lang="en-ZA" sz="1100"/>
+                  <a:t>This shape represents a slicer. Slicers are supported in Excel 2010 or later.
+If the shape was modified in an earlier version of Excel, or if the workbook was saved in Excel 2003 or earlier, the slicer cannot be used.</a:t>
+                </a:r>
+              </a:p>
+            </xdr:txBody>
+          </xdr:sp>
+        </mc:Fallback>
+      </mc:AlternateContent>
+      <xdr:sp macro="" textlink="">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="2" name="Rectangle 1">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDF370E7-A90F-4DAE-B746-ADE9B571236B}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="7388" y="4529005"/>
+            <a:ext cx="4288035" cy="489113"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="accent5">
+              <a:lumMod val="60000"/>
+              <a:lumOff val="40000"/>
+            </a:schemeClr>
+          </a:solidFill>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-ZA" sz="2800" b="1" u="none">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+              </a:rPr>
+              <a:t>Filter By:</a:t>
+            </a:r>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>613076</xdr:colOff>
-      <xdr:row>3</xdr:row>
-      <xdr:rowOff>38069</xdr:rowOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>590082</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>118363</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>17517</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>8760</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Rectangle 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{EDF370E7-A90F-4DAE-B746-ADE9B571236B}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18393076" y="589862"/>
-          <a:ext cx="4309269" cy="522484"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="accent5">
-            <a:lumMod val="60000"/>
-            <a:lumOff val="40000"/>
-          </a:schemeClr>
-        </a:solidFill>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-ZA" sz="2800" b="1" u="none">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-            </a:rPr>
-            <a:t>FILTER BY:</a:t>
-          </a:r>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>611</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>162275</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>14111</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>172720</xdr:rowOff>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>603583</xdr:colOff>
+      <xdr:row>52</xdr:row>
+      <xdr:rowOff>182408</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8566,16 +9161,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>4134</xdr:colOff>
+      <xdr:col>27</xdr:col>
+      <xdr:colOff>593605</xdr:colOff>
       <xdr:row>25</xdr:row>
-      <xdr:rowOff>13874</xdr:rowOff>
+      <xdr:rowOff>160463</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>10160</xdr:colOff>
-      <xdr:row>27</xdr:row>
-      <xdr:rowOff>162012</xdr:rowOff>
+      <xdr:col>41</xdr:col>
+      <xdr:colOff>599632</xdr:colOff>
+      <xdr:row>28</xdr:row>
+      <xdr:rowOff>118101</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
@@ -8590,8 +9185,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="9148134" y="4585874"/>
-          <a:ext cx="8540426" cy="513898"/>
+          <a:off x="16897530" y="4833105"/>
+          <a:ext cx="8459913" cy="518354"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -8639,336 +9234,16 @@
   </xdr:twoCellAnchor>
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>7903</xdr:colOff>
-      <xdr:row>33</xdr:row>
-      <xdr:rowOff>17152</xdr:rowOff>
+      <xdr:col>32</xdr:col>
+      <xdr:colOff>585063</xdr:colOff>
+      <xdr:row>6</xdr:row>
+      <xdr:rowOff>168751</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>37</xdr:row>
-      <xdr:rowOff>170330</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="Pivot_Tables!F4">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="21" name="Rectangle 20">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{814B24ED-8E5A-6ED0-D234-BE30BA85FF30}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18295903" y="5933858"/>
-          <a:ext cx="4259297" cy="870354"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="accent5">
-              <a:lumMod val="60000"/>
-              <a:lumOff val="40000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:t>Total</a:t>
-          </a:r>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike" baseline="0">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:t> Revenue</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:fld id="{1487D781-EC85-44F9-BD03-BF5F1C979E13}" type="TxLink">
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:sysClr val="windowText" lastClr="000000"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:pPr algn="ctr"/>
-            <a:t>R903 500</a:t>
-          </a:fld>
-          <a:endParaRPr lang="en-ZA" sz="2000" b="1">
-            <a:solidFill>
-              <a:sysClr val="windowText" lastClr="000000"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>3267</xdr:colOff>
-      <xdr:row>38</xdr:row>
-      <xdr:rowOff>12070</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>8965</xdr:colOff>
-      <xdr:row>42</xdr:row>
-      <xdr:rowOff>170329</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="Pivot_Tables!F7">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="24" name="Rectangle 23">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0CD2E6D-C1F9-48F7-B1F6-04B40FA69F9F}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18291267" y="6825246"/>
-          <a:ext cx="4272898" cy="875436"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="accent5">
-              <a:lumMod val="60000"/>
-              <a:lumOff val="40000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:t>Total Quantity</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:fld id="{A2CC588B-4206-4FEE-94FC-AA5B2B8DB377}" type="TxLink">
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:pPr algn="ctr"/>
-            <a:t>159</a:t>
-          </a:fld>
-          <a:endParaRPr lang="en-ZA" sz="2000" b="1">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>30</xdr:col>
-      <xdr:colOff>13133</xdr:colOff>
-      <xdr:row>43</xdr:row>
-      <xdr:rowOff>17771</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>37</xdr:col>
-      <xdr:colOff>8964</xdr:colOff>
-      <xdr:row>47</xdr:row>
-      <xdr:rowOff>170329</xdr:rowOff>
-    </xdr:to>
-    <xdr:sp macro="" textlink="Pivot_Tables!F13">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="28" name="Rectangle 27">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9BA0F6C1-E535-46A5-BCF3-7EF50A1833D5}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="18301133" y="7727418"/>
-          <a:ext cx="4263031" cy="869735"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:solidFill>
-          <a:schemeClr val="bg1">
-            <a:lumMod val="85000"/>
-          </a:schemeClr>
-        </a:solidFill>
-        <a:ln>
-          <a:solidFill>
-            <a:schemeClr val="accent5">
-              <a:lumMod val="60000"/>
-              <a:lumOff val="40000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1">
-            <a:shade val="15000"/>
-          </a:schemeClr>
-        </a:lnRef>
-        <a:fillRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="lt1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
-        <a:lstStyle/>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:r>
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:t>Top Product</a:t>
-          </a:r>
-        </a:p>
-        <a:p>
-          <a:pPr algn="ctr"/>
-          <a:fld id="{7F136A86-B18F-4AAA-95D5-73628CBD541F}" type="TxLink">
-            <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
-              <a:solidFill>
-                <a:schemeClr val="tx1"/>
-              </a:solidFill>
-              <a:latin typeface="Calibri"/>
-              <a:ea typeface="Calibri"/>
-              <a:cs typeface="Calibri"/>
-            </a:rPr>
-            <a:pPr algn="ctr"/>
-            <a:t>Phone</a:t>
-          </a:fld>
-          <a:endParaRPr lang="en-ZA" sz="2000" b="1">
-            <a:solidFill>
-              <a:schemeClr val="tx1"/>
-            </a:solidFill>
-          </a:endParaRPr>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>19</xdr:col>
-      <xdr:colOff>550418</xdr:colOff>
-      <xdr:row>6</xdr:row>
-      <xdr:rowOff>25756</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>29</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
-      <xdr:row>22</xdr:row>
-      <xdr:rowOff>157654</xdr:rowOff>
+      <xdr:col>42</xdr:col>
+      <xdr:colOff>16103</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>113743</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -8991,6 +9266,421 @@
         </a:graphicData>
       </a:graphic>
     </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>589474</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>186424</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>595171</xdr:colOff>
+      <xdr:row>23</xdr:row>
+      <xdr:rowOff>19151</xdr:rowOff>
+    </xdr:to>
+    <xdr:grpSp>
+      <xdr:nvGrpSpPr>
+        <xdr:cNvPr id="10" name="Group 9">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{30E6B6D0-D054-361A-73E0-33D35ADDCD6F}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvGrpSpPr/>
+      </xdr:nvGrpSpPr>
+      <xdr:grpSpPr>
+        <a:xfrm>
+          <a:off x="3008522" y="730710"/>
+          <a:ext cx="4239030" cy="3461298"/>
+          <a:chOff x="2" y="769553"/>
+          <a:chExt cx="4232641" cy="3570840"/>
+        </a:xfrm>
+      </xdr:grpSpPr>
+      <xdr:sp macro="" textlink="Pivot_Tables!F4">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="21" name="Rectangle 20">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{814B24ED-8E5A-6ED0-D234-BE30BA85FF30}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="4677" y="769553"/>
+            <a:ext cx="4222386" cy="1220833"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="95000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Total</a:t>
+            </a:r>
+            <a:r>
+              <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike" baseline="0">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:t> Revenue </a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:fld id="{1487D781-EC85-44F9-BD03-BF5F1C979E13}" type="TxLink">
+              <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:sysClr val="windowText" lastClr="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:pPr algn="ctr"/>
+              <a:t>R903 500</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-ZA" sz="2000" b="1">
+              <a:solidFill>
+                <a:sysClr val="windowText" lastClr="000000"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="Pivot_Tables!F7">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="24" name="Rectangle 23">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{F0CD2E6D-C1F9-48F7-B1F6-04B40FA69F9F}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="2" y="1878990"/>
+            <a:ext cx="4232641" cy="1227577"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="95000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Total Quantity</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:fld id="{A2CC588B-4206-4FEE-94FC-AA5B2B8DB377}" type="TxLink">
+              <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:pPr algn="ctr"/>
+              <a:t>159</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-ZA" sz="2000" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:sp macro="" textlink="Pivot_Tables!F13">
+        <xdr:nvSpPr>
+          <xdr:cNvPr id="28" name="Rectangle 27">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9BA0F6C1-E535-46A5-BCF3-7EF50A1833D5}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvSpPr/>
+        </xdr:nvSpPr>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="9952" y="3113585"/>
+            <a:ext cx="4222688" cy="1226808"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+          <a:solidFill>
+            <a:schemeClr val="bg1">
+              <a:lumMod val="95000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:ln>
+            <a:solidFill>
+              <a:schemeClr val="accent5">
+                <a:lumMod val="60000"/>
+                <a:lumOff val="40000"/>
+              </a:schemeClr>
+            </a:solidFill>
+          </a:ln>
+        </xdr:spPr>
+        <xdr:style>
+          <a:lnRef idx="2">
+            <a:schemeClr val="accent1">
+              <a:shade val="15000"/>
+            </a:schemeClr>
+          </a:lnRef>
+          <a:fillRef idx="1">
+            <a:schemeClr val="accent1"/>
+          </a:fillRef>
+          <a:effectRef idx="0">
+            <a:schemeClr val="accent1"/>
+          </a:effectRef>
+          <a:fontRef idx="minor">
+            <a:schemeClr val="lt1"/>
+          </a:fontRef>
+        </xdr:style>
+        <xdr:txBody>
+          <a:bodyPr vertOverflow="clip" horzOverflow="clip" rtlCol="0" anchor="ctr"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:r>
+              <a:rPr lang="en-US" sz="2000" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Top Product</a:t>
+            </a:r>
+          </a:p>
+          <a:p>
+            <a:pPr algn="ctr"/>
+            <a:fld id="{7F136A86-B18F-4AAA-95D5-73628CBD541F}" type="TxLink">
+              <a:rPr lang="en-US" sz="3200" b="1" i="0" u="none" strike="noStrike">
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+                <a:ea typeface="Calibri"/>
+                <a:cs typeface="Calibri"/>
+              </a:rPr>
+              <a:pPr algn="ctr"/>
+              <a:t>Phone</a:t>
+            </a:fld>
+            <a:endParaRPr lang="en-ZA" sz="2000" b="1">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:endParaRPr>
+          </a:p>
+        </xdr:txBody>
+      </xdr:sp>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="30" name="Picture 29">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DFBCD78B-77C2-DA48-57D0-8F4EFABC2597}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId8" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3527246" y="1145569"/>
+            <a:ext cx="657322" cy="667411"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="32" name="Picture 31">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{B878F728-F11E-30DD-6827-E09CC3157839}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId9" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3580719" y="2354275"/>
+            <a:ext cx="617218" cy="627307"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+      <xdr:pic>
+        <xdr:nvPicPr>
+          <xdr:cNvPr id="34" name="Picture 33">
+            <a:extLst>
+              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{9FD191F8-C8DB-596A-3142-3938E68BE8AD}"/>
+              </a:ext>
+            </a:extLst>
+          </xdr:cNvPr>
+          <xdr:cNvPicPr>
+            <a:picLocks noChangeAspect="1"/>
+          </xdr:cNvPicPr>
+        </xdr:nvPicPr>
+        <xdr:blipFill>
+          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId10" cstate="print">
+            <a:extLst>
+              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+              </a:ext>
+            </a:extLst>
+          </a:blip>
+          <a:stretch>
+            <a:fillRect/>
+          </a:stretch>
+        </xdr:blipFill>
+        <xdr:spPr>
+          <a:xfrm>
+            <a:off x="3549924" y="3568210"/>
+            <a:ext cx="661620" cy="694539"/>
+          </a:xfrm>
+          <a:prstGeom prst="rect">
+            <a:avLst/>
+          </a:prstGeom>
+        </xdr:spPr>
+      </xdr:pic>
+    </xdr:grpSp>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -10045,7 +10735,108 @@
 </file>
 
 <file path=xl/pivotTables/pivotTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EF61005-3DC2-4F04-A889-30AB3AB0D1A3}" name="Salesperson Performance Monthly" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="16">
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A92E6C64-2F9D-443D-AE81-1304DED4A368}" name="Saleperson Performance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
+  <location ref="A29:B35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0" defaultSubtotal="0"/>
+    <pivotField showAll="0" defaultSubtotal="0">
+      <items count="14">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="7"/>
+  </rowFields>
+  <rowItems count="6">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i>
+      <x v="4"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
+  </dataFields>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{1EF61005-3DC2-4F04-A889-30AB3AB0D1A3}" name="Salesperson Performance Monthly" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="24">
   <location ref="A64:F73" firstHeaderRow="1" firstDataRow="4" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -10713,8 +11504,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable2.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2EBA4ED6-0263-4163-B60D-94E9DAE81843}" name="Product Category Distribution" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="29">
+<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{2EBA4ED6-0263-4163-B60D-94E9DAE81843}" name="Product Category Distribution" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="33">
   <location ref="A39:B50" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -10930,7 +11721,503 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F701EDC3-81C2-4D13-8691-DB7E36575968}" name="Sales by Region" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
+  <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
+  <pivotFields count="12">
+    <pivotField showAll="0"/>
+    <pivotField numFmtId="14" showAll="0"/>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="4"/>
+        <item x="3"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="3">
+        <item x="0"/>
+        <item x="1"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0"/>
+    <pivotField showAll="0"/>
+    <pivotField axis="axisRow" showAll="0">
+      <items count="5">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="6">
+        <item x="2"/>
+        <item x="0"/>
+        <item x="1"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField dataField="1" showAll="0"/>
+    <pivotField numFmtId="14" showAll="0">
+      <items count="5">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="369">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item x="14"/>
+        <item x="15"/>
+        <item x="16"/>
+        <item x="17"/>
+        <item x="18"/>
+        <item x="19"/>
+        <item x="20"/>
+        <item x="21"/>
+        <item x="22"/>
+        <item x="23"/>
+        <item x="24"/>
+        <item x="25"/>
+        <item x="26"/>
+        <item x="27"/>
+        <item x="28"/>
+        <item x="29"/>
+        <item x="30"/>
+        <item x="31"/>
+        <item x="32"/>
+        <item x="33"/>
+        <item x="34"/>
+        <item x="35"/>
+        <item x="36"/>
+        <item x="37"/>
+        <item x="38"/>
+        <item x="39"/>
+        <item x="40"/>
+        <item x="41"/>
+        <item x="42"/>
+        <item x="43"/>
+        <item x="44"/>
+        <item x="45"/>
+        <item x="46"/>
+        <item x="47"/>
+        <item x="48"/>
+        <item x="49"/>
+        <item x="50"/>
+        <item x="51"/>
+        <item x="52"/>
+        <item x="53"/>
+        <item x="54"/>
+        <item x="55"/>
+        <item x="56"/>
+        <item x="57"/>
+        <item x="58"/>
+        <item x="59"/>
+        <item x="60"/>
+        <item x="61"/>
+        <item x="62"/>
+        <item x="63"/>
+        <item x="64"/>
+        <item x="65"/>
+        <item x="66"/>
+        <item x="67"/>
+        <item x="68"/>
+        <item x="69"/>
+        <item x="70"/>
+        <item x="71"/>
+        <item x="72"/>
+        <item x="73"/>
+        <item x="74"/>
+        <item x="75"/>
+        <item x="76"/>
+        <item x="77"/>
+        <item x="78"/>
+        <item x="79"/>
+        <item x="80"/>
+        <item x="81"/>
+        <item x="82"/>
+        <item x="83"/>
+        <item x="84"/>
+        <item x="85"/>
+        <item x="86"/>
+        <item x="87"/>
+        <item x="88"/>
+        <item x="89"/>
+        <item x="90"/>
+        <item x="91"/>
+        <item x="92"/>
+        <item x="93"/>
+        <item x="94"/>
+        <item x="95"/>
+        <item x="96"/>
+        <item x="97"/>
+        <item x="98"/>
+        <item x="99"/>
+        <item x="100"/>
+        <item x="101"/>
+        <item x="102"/>
+        <item x="103"/>
+        <item x="104"/>
+        <item x="105"/>
+        <item x="106"/>
+        <item x="107"/>
+        <item x="108"/>
+        <item x="109"/>
+        <item x="110"/>
+        <item x="111"/>
+        <item x="112"/>
+        <item x="113"/>
+        <item x="114"/>
+        <item x="115"/>
+        <item x="116"/>
+        <item x="117"/>
+        <item x="118"/>
+        <item x="119"/>
+        <item x="120"/>
+        <item x="121"/>
+        <item x="122"/>
+        <item x="123"/>
+        <item x="124"/>
+        <item x="125"/>
+        <item x="126"/>
+        <item x="127"/>
+        <item x="128"/>
+        <item x="129"/>
+        <item x="130"/>
+        <item x="131"/>
+        <item x="132"/>
+        <item x="133"/>
+        <item x="134"/>
+        <item x="135"/>
+        <item x="136"/>
+        <item x="137"/>
+        <item x="138"/>
+        <item x="139"/>
+        <item x="140"/>
+        <item x="141"/>
+        <item x="142"/>
+        <item x="143"/>
+        <item x="144"/>
+        <item x="145"/>
+        <item x="146"/>
+        <item x="147"/>
+        <item x="148"/>
+        <item x="149"/>
+        <item x="150"/>
+        <item x="151"/>
+        <item x="152"/>
+        <item x="153"/>
+        <item x="154"/>
+        <item x="155"/>
+        <item x="156"/>
+        <item x="157"/>
+        <item x="158"/>
+        <item x="159"/>
+        <item x="160"/>
+        <item x="161"/>
+        <item x="162"/>
+        <item x="163"/>
+        <item x="164"/>
+        <item x="165"/>
+        <item x="166"/>
+        <item x="167"/>
+        <item x="168"/>
+        <item x="169"/>
+        <item x="170"/>
+        <item x="171"/>
+        <item x="172"/>
+        <item x="173"/>
+        <item x="174"/>
+        <item x="175"/>
+        <item x="176"/>
+        <item x="177"/>
+        <item x="178"/>
+        <item x="179"/>
+        <item x="180"/>
+        <item x="181"/>
+        <item x="182"/>
+        <item x="183"/>
+        <item x="184"/>
+        <item x="185"/>
+        <item x="186"/>
+        <item x="187"/>
+        <item x="188"/>
+        <item x="189"/>
+        <item x="190"/>
+        <item x="191"/>
+        <item x="192"/>
+        <item x="193"/>
+        <item x="194"/>
+        <item x="195"/>
+        <item x="196"/>
+        <item x="197"/>
+        <item x="198"/>
+        <item x="199"/>
+        <item x="200"/>
+        <item x="201"/>
+        <item x="202"/>
+        <item x="203"/>
+        <item x="204"/>
+        <item x="205"/>
+        <item x="206"/>
+        <item x="207"/>
+        <item x="208"/>
+        <item x="209"/>
+        <item x="210"/>
+        <item x="211"/>
+        <item x="212"/>
+        <item x="213"/>
+        <item x="214"/>
+        <item x="215"/>
+        <item x="216"/>
+        <item x="217"/>
+        <item x="218"/>
+        <item x="219"/>
+        <item x="220"/>
+        <item x="221"/>
+        <item x="222"/>
+        <item x="223"/>
+        <item x="224"/>
+        <item x="225"/>
+        <item x="226"/>
+        <item x="227"/>
+        <item x="228"/>
+        <item x="229"/>
+        <item x="230"/>
+        <item x="231"/>
+        <item x="232"/>
+        <item x="233"/>
+        <item x="234"/>
+        <item x="235"/>
+        <item x="236"/>
+        <item x="237"/>
+        <item x="238"/>
+        <item x="239"/>
+        <item x="240"/>
+        <item x="241"/>
+        <item x="242"/>
+        <item x="243"/>
+        <item x="244"/>
+        <item x="245"/>
+        <item x="246"/>
+        <item x="247"/>
+        <item x="248"/>
+        <item x="249"/>
+        <item x="250"/>
+        <item x="251"/>
+        <item x="252"/>
+        <item x="253"/>
+        <item x="254"/>
+        <item x="255"/>
+        <item x="256"/>
+        <item x="257"/>
+        <item x="258"/>
+        <item x="259"/>
+        <item x="260"/>
+        <item x="261"/>
+        <item x="262"/>
+        <item x="263"/>
+        <item x="264"/>
+        <item x="265"/>
+        <item x="266"/>
+        <item x="267"/>
+        <item x="268"/>
+        <item x="269"/>
+        <item x="270"/>
+        <item x="271"/>
+        <item x="272"/>
+        <item x="273"/>
+        <item x="274"/>
+        <item x="275"/>
+        <item x="276"/>
+        <item x="277"/>
+        <item x="278"/>
+        <item x="279"/>
+        <item x="280"/>
+        <item x="281"/>
+        <item x="282"/>
+        <item x="283"/>
+        <item x="284"/>
+        <item x="285"/>
+        <item x="286"/>
+        <item x="287"/>
+        <item x="288"/>
+        <item x="289"/>
+        <item x="290"/>
+        <item x="291"/>
+        <item x="292"/>
+        <item x="293"/>
+        <item x="294"/>
+        <item x="295"/>
+        <item x="296"/>
+        <item x="297"/>
+        <item x="298"/>
+        <item x="299"/>
+        <item x="300"/>
+        <item x="301"/>
+        <item x="302"/>
+        <item x="303"/>
+        <item x="304"/>
+        <item x="305"/>
+        <item x="306"/>
+        <item x="307"/>
+        <item x="308"/>
+        <item x="309"/>
+        <item x="310"/>
+        <item x="311"/>
+        <item x="312"/>
+        <item x="313"/>
+        <item x="314"/>
+        <item x="315"/>
+        <item x="316"/>
+        <item x="317"/>
+        <item x="318"/>
+        <item x="319"/>
+        <item x="320"/>
+        <item x="321"/>
+        <item x="322"/>
+        <item x="323"/>
+        <item x="324"/>
+        <item x="325"/>
+        <item x="326"/>
+        <item x="327"/>
+        <item x="328"/>
+        <item x="329"/>
+        <item x="330"/>
+        <item x="331"/>
+        <item x="332"/>
+        <item x="333"/>
+        <item x="334"/>
+        <item x="335"/>
+        <item x="336"/>
+        <item x="337"/>
+        <item x="338"/>
+        <item x="339"/>
+        <item x="340"/>
+        <item x="341"/>
+        <item x="342"/>
+        <item x="343"/>
+        <item x="344"/>
+        <item x="345"/>
+        <item x="346"/>
+        <item x="347"/>
+        <item x="348"/>
+        <item x="349"/>
+        <item x="350"/>
+        <item x="351"/>
+        <item x="352"/>
+        <item x="353"/>
+        <item x="354"/>
+        <item x="355"/>
+        <item x="356"/>
+        <item x="357"/>
+        <item x="358"/>
+        <item x="359"/>
+        <item x="360"/>
+        <item x="361"/>
+        <item x="362"/>
+        <item x="363"/>
+        <item x="364"/>
+        <item x="365"/>
+        <item x="366"/>
+        <item x="367"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+    <pivotField showAll="0">
+      <items count="15">
+        <item x="0"/>
+        <item x="1"/>
+        <item x="2"/>
+        <item x="3"/>
+        <item x="4"/>
+        <item x="5"/>
+        <item x="6"/>
+        <item x="7"/>
+        <item x="8"/>
+        <item x="9"/>
+        <item x="10"/>
+        <item x="11"/>
+        <item x="12"/>
+        <item x="13"/>
+        <item t="default"/>
+      </items>
+    </pivotField>
+  </pivotFields>
+  <rowFields count="1">
+    <field x="6"/>
+  </rowFields>
+  <rowItems count="5">
+    <i>
+      <x/>
+    </i>
+    <i>
+      <x v="1"/>
+    </i>
+    <i>
+      <x v="2"/>
+    </i>
+    <i>
+      <x v="3"/>
+    </i>
+    <i t="grand">
+      <x/>
+    </i>
+  </rowItems>
+  <colItems count="1">
+    <i/>
+  </colItems>
+  <dataFields count="1">
+    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
+  </dataFields>
+  <chartFormats count="1">
+    <chartFormat chart="2" format="1" series="1">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="1">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+  </chartFormats>
+  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
+      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
+    </ext>
+    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
+      <xpdl:pivotTableDefinition16/>
+    </ext>
+  </extLst>
+</pivotTableDefinition>
+</file>
+
+<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{EEA1BD0D-A2BA-41BA-AC63-F069DCA73CCD}" name="Monthly Revenue Trends" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="8">
   <location ref="A20:B25" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
@@ -11428,7 +12715,7 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
 <pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{77BF86ED-9B5C-443E-BA35-5E459117CD3F}" name="Top Performing Products" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
   <location ref="A10:B16" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
   <pivotFields count="12">
@@ -11985,8 +13272,8 @@
 </pivotTableDefinition>
 </file>
 
-<file path=xl/pivotTables/pivotTable5.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C975136F-C808-4BF6-9947-A39165D24CB0}" name="Products of the Month" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="11">
+<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
+<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{C975136F-C808-4BF6-9947-A39165D24CB0}" name="Products of the Month" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="15">
   <location ref="A54:G60" firstHeaderRow="1" firstDataRow="2" firstDataCol="1"/>
   <pivotFields count="12">
     <pivotField showAll="0"/>
@@ -12478,7 +13765,7 @@
   <dataFields count="1">
     <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
   </dataFields>
-  <chartFormats count="6">
+  <chartFormats count="8">
     <chartFormat chart="2" format="5" series="1">
       <pivotArea type="data" outline="0" fieldPosition="0">
         <references count="2">
@@ -12548,599 +13835,32 @@
         </references>
       </pivotArea>
     </chartFormat>
-  </chartFormats>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable6.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{A92E6C64-2F9D-443D-AE81-1304DED4A368}" name="Saleperson Performance" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0">
-  <location ref="A29:B35" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="4"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0" defaultSubtotal="0"/>
-    <pivotField showAll="0" defaultSubtotal="0">
-      <items count="14">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="7"/>
-  </rowFields>
-  <rowItems count="6">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i>
-      <x v="4"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
-  </dataFields>
-  <pivotTableStyleInfo name="PivotStyleLight16" showRowHeaders="1" showColHeaders="1" showRowStripes="0" showColStripes="0" showLastColumn="1"/>
-  <extLst>
-    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{962EF5D1-5CA2-4c93-8EF4-DBF5C05439D2}">
-      <x14:pivotTableDefinition xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" hideValuesRow="1"/>
-    </ext>
-    <ext xmlns:xpdl="http://schemas.microsoft.com/office/spreadsheetml/2016/pivotdefaultlayout" uri="{747A6164-185A-40DC-8AA5-F01512510D54}">
-      <xpdl:pivotTableDefinition16/>
-    </ext>
-  </extLst>
-</pivotTableDefinition>
-</file>
-
-<file path=xl/pivotTables/pivotTable7.xml><?xml version="1.0" encoding="utf-8"?>
-<pivotTableDefinition xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr" xr:uid="{F701EDC3-81C2-4D13-8691-DB7E36575968}" name="Sales by Region" cacheId="0" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="1" dataCaption="Values" updatedVersion="8" minRefreshableVersion="5" useAutoFormatting="1" itemPrintTitles="1" createdVersion="8" indent="0" outline="1" outlineData="1" multipleFieldFilters="0" chartFormat="7">
-  <location ref="A1:B6" firstHeaderRow="1" firstDataRow="1" firstDataCol="1"/>
-  <pivotFields count="12">
-    <pivotField showAll="0"/>
-    <pivotField numFmtId="14" showAll="0"/>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="4"/>
-        <item x="3"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="3">
-        <item x="0"/>
-        <item x="1"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0"/>
-    <pivotField showAll="0"/>
-    <pivotField axis="axisRow" showAll="0">
-      <items count="5">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="6">
-        <item x="2"/>
-        <item x="0"/>
-        <item x="1"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField dataField="1" showAll="0"/>
-    <pivotField numFmtId="14" showAll="0">
-      <items count="5">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="369">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item x="14"/>
-        <item x="15"/>
-        <item x="16"/>
-        <item x="17"/>
-        <item x="18"/>
-        <item x="19"/>
-        <item x="20"/>
-        <item x="21"/>
-        <item x="22"/>
-        <item x="23"/>
-        <item x="24"/>
-        <item x="25"/>
-        <item x="26"/>
-        <item x="27"/>
-        <item x="28"/>
-        <item x="29"/>
-        <item x="30"/>
-        <item x="31"/>
-        <item x="32"/>
-        <item x="33"/>
-        <item x="34"/>
-        <item x="35"/>
-        <item x="36"/>
-        <item x="37"/>
-        <item x="38"/>
-        <item x="39"/>
-        <item x="40"/>
-        <item x="41"/>
-        <item x="42"/>
-        <item x="43"/>
-        <item x="44"/>
-        <item x="45"/>
-        <item x="46"/>
-        <item x="47"/>
-        <item x="48"/>
-        <item x="49"/>
-        <item x="50"/>
-        <item x="51"/>
-        <item x="52"/>
-        <item x="53"/>
-        <item x="54"/>
-        <item x="55"/>
-        <item x="56"/>
-        <item x="57"/>
-        <item x="58"/>
-        <item x="59"/>
-        <item x="60"/>
-        <item x="61"/>
-        <item x="62"/>
-        <item x="63"/>
-        <item x="64"/>
-        <item x="65"/>
-        <item x="66"/>
-        <item x="67"/>
-        <item x="68"/>
-        <item x="69"/>
-        <item x="70"/>
-        <item x="71"/>
-        <item x="72"/>
-        <item x="73"/>
-        <item x="74"/>
-        <item x="75"/>
-        <item x="76"/>
-        <item x="77"/>
-        <item x="78"/>
-        <item x="79"/>
-        <item x="80"/>
-        <item x="81"/>
-        <item x="82"/>
-        <item x="83"/>
-        <item x="84"/>
-        <item x="85"/>
-        <item x="86"/>
-        <item x="87"/>
-        <item x="88"/>
-        <item x="89"/>
-        <item x="90"/>
-        <item x="91"/>
-        <item x="92"/>
-        <item x="93"/>
-        <item x="94"/>
-        <item x="95"/>
-        <item x="96"/>
-        <item x="97"/>
-        <item x="98"/>
-        <item x="99"/>
-        <item x="100"/>
-        <item x="101"/>
-        <item x="102"/>
-        <item x="103"/>
-        <item x="104"/>
-        <item x="105"/>
-        <item x="106"/>
-        <item x="107"/>
-        <item x="108"/>
-        <item x="109"/>
-        <item x="110"/>
-        <item x="111"/>
-        <item x="112"/>
-        <item x="113"/>
-        <item x="114"/>
-        <item x="115"/>
-        <item x="116"/>
-        <item x="117"/>
-        <item x="118"/>
-        <item x="119"/>
-        <item x="120"/>
-        <item x="121"/>
-        <item x="122"/>
-        <item x="123"/>
-        <item x="124"/>
-        <item x="125"/>
-        <item x="126"/>
-        <item x="127"/>
-        <item x="128"/>
-        <item x="129"/>
-        <item x="130"/>
-        <item x="131"/>
-        <item x="132"/>
-        <item x="133"/>
-        <item x="134"/>
-        <item x="135"/>
-        <item x="136"/>
-        <item x="137"/>
-        <item x="138"/>
-        <item x="139"/>
-        <item x="140"/>
-        <item x="141"/>
-        <item x="142"/>
-        <item x="143"/>
-        <item x="144"/>
-        <item x="145"/>
-        <item x="146"/>
-        <item x="147"/>
-        <item x="148"/>
-        <item x="149"/>
-        <item x="150"/>
-        <item x="151"/>
-        <item x="152"/>
-        <item x="153"/>
-        <item x="154"/>
-        <item x="155"/>
-        <item x="156"/>
-        <item x="157"/>
-        <item x="158"/>
-        <item x="159"/>
-        <item x="160"/>
-        <item x="161"/>
-        <item x="162"/>
-        <item x="163"/>
-        <item x="164"/>
-        <item x="165"/>
-        <item x="166"/>
-        <item x="167"/>
-        <item x="168"/>
-        <item x="169"/>
-        <item x="170"/>
-        <item x="171"/>
-        <item x="172"/>
-        <item x="173"/>
-        <item x="174"/>
-        <item x="175"/>
-        <item x="176"/>
-        <item x="177"/>
-        <item x="178"/>
-        <item x="179"/>
-        <item x="180"/>
-        <item x="181"/>
-        <item x="182"/>
-        <item x="183"/>
-        <item x="184"/>
-        <item x="185"/>
-        <item x="186"/>
-        <item x="187"/>
-        <item x="188"/>
-        <item x="189"/>
-        <item x="190"/>
-        <item x="191"/>
-        <item x="192"/>
-        <item x="193"/>
-        <item x="194"/>
-        <item x="195"/>
-        <item x="196"/>
-        <item x="197"/>
-        <item x="198"/>
-        <item x="199"/>
-        <item x="200"/>
-        <item x="201"/>
-        <item x="202"/>
-        <item x="203"/>
-        <item x="204"/>
-        <item x="205"/>
-        <item x="206"/>
-        <item x="207"/>
-        <item x="208"/>
-        <item x="209"/>
-        <item x="210"/>
-        <item x="211"/>
-        <item x="212"/>
-        <item x="213"/>
-        <item x="214"/>
-        <item x="215"/>
-        <item x="216"/>
-        <item x="217"/>
-        <item x="218"/>
-        <item x="219"/>
-        <item x="220"/>
-        <item x="221"/>
-        <item x="222"/>
-        <item x="223"/>
-        <item x="224"/>
-        <item x="225"/>
-        <item x="226"/>
-        <item x="227"/>
-        <item x="228"/>
-        <item x="229"/>
-        <item x="230"/>
-        <item x="231"/>
-        <item x="232"/>
-        <item x="233"/>
-        <item x="234"/>
-        <item x="235"/>
-        <item x="236"/>
-        <item x="237"/>
-        <item x="238"/>
-        <item x="239"/>
-        <item x="240"/>
-        <item x="241"/>
-        <item x="242"/>
-        <item x="243"/>
-        <item x="244"/>
-        <item x="245"/>
-        <item x="246"/>
-        <item x="247"/>
-        <item x="248"/>
-        <item x="249"/>
-        <item x="250"/>
-        <item x="251"/>
-        <item x="252"/>
-        <item x="253"/>
-        <item x="254"/>
-        <item x="255"/>
-        <item x="256"/>
-        <item x="257"/>
-        <item x="258"/>
-        <item x="259"/>
-        <item x="260"/>
-        <item x="261"/>
-        <item x="262"/>
-        <item x="263"/>
-        <item x="264"/>
-        <item x="265"/>
-        <item x="266"/>
-        <item x="267"/>
-        <item x="268"/>
-        <item x="269"/>
-        <item x="270"/>
-        <item x="271"/>
-        <item x="272"/>
-        <item x="273"/>
-        <item x="274"/>
-        <item x="275"/>
-        <item x="276"/>
-        <item x="277"/>
-        <item x="278"/>
-        <item x="279"/>
-        <item x="280"/>
-        <item x="281"/>
-        <item x="282"/>
-        <item x="283"/>
-        <item x="284"/>
-        <item x="285"/>
-        <item x="286"/>
-        <item x="287"/>
-        <item x="288"/>
-        <item x="289"/>
-        <item x="290"/>
-        <item x="291"/>
-        <item x="292"/>
-        <item x="293"/>
-        <item x="294"/>
-        <item x="295"/>
-        <item x="296"/>
-        <item x="297"/>
-        <item x="298"/>
-        <item x="299"/>
-        <item x="300"/>
-        <item x="301"/>
-        <item x="302"/>
-        <item x="303"/>
-        <item x="304"/>
-        <item x="305"/>
-        <item x="306"/>
-        <item x="307"/>
-        <item x="308"/>
-        <item x="309"/>
-        <item x="310"/>
-        <item x="311"/>
-        <item x="312"/>
-        <item x="313"/>
-        <item x="314"/>
-        <item x="315"/>
-        <item x="316"/>
-        <item x="317"/>
-        <item x="318"/>
-        <item x="319"/>
-        <item x="320"/>
-        <item x="321"/>
-        <item x="322"/>
-        <item x="323"/>
-        <item x="324"/>
-        <item x="325"/>
-        <item x="326"/>
-        <item x="327"/>
-        <item x="328"/>
-        <item x="329"/>
-        <item x="330"/>
-        <item x="331"/>
-        <item x="332"/>
-        <item x="333"/>
-        <item x="334"/>
-        <item x="335"/>
-        <item x="336"/>
-        <item x="337"/>
-        <item x="338"/>
-        <item x="339"/>
-        <item x="340"/>
-        <item x="341"/>
-        <item x="342"/>
-        <item x="343"/>
-        <item x="344"/>
-        <item x="345"/>
-        <item x="346"/>
-        <item x="347"/>
-        <item x="348"/>
-        <item x="349"/>
-        <item x="350"/>
-        <item x="351"/>
-        <item x="352"/>
-        <item x="353"/>
-        <item x="354"/>
-        <item x="355"/>
-        <item x="356"/>
-        <item x="357"/>
-        <item x="358"/>
-        <item x="359"/>
-        <item x="360"/>
-        <item x="361"/>
-        <item x="362"/>
-        <item x="363"/>
-        <item x="364"/>
-        <item x="365"/>
-        <item x="366"/>
-        <item x="367"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-    <pivotField showAll="0">
-      <items count="15">
-        <item x="0"/>
-        <item x="1"/>
-        <item x="2"/>
-        <item x="3"/>
-        <item x="4"/>
-        <item x="5"/>
-        <item x="6"/>
-        <item x="7"/>
-        <item x="8"/>
-        <item x="9"/>
-        <item x="10"/>
-        <item x="11"/>
-        <item x="12"/>
-        <item x="13"/>
-        <item t="default"/>
-      </items>
-    </pivotField>
-  </pivotFields>
-  <rowFields count="1">
-    <field x="6"/>
-  </rowFields>
-  <rowItems count="5">
-    <i>
-      <x/>
-    </i>
-    <i>
-      <x v="1"/>
-    </i>
-    <i>
-      <x v="2"/>
-    </i>
-    <i>
-      <x v="3"/>
-    </i>
-    <i t="grand">
-      <x/>
-    </i>
-  </rowItems>
-  <colItems count="1">
-    <i/>
-  </colItems>
-  <dataFields count="1">
-    <dataField name="Sum of revenue" fld="8" baseField="0" baseItem="0"/>
-  </dataFields>
-  <chartFormats count="1">
-    <chartFormat chart="2" format="1" series="1">
+    <chartFormat chart="2" format="11">
       <pivotArea type="data" outline="0" fieldPosition="0">
-        <references count="1">
+        <references count="3">
           <reference field="4294967294" count="1" selected="0">
             <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="11" count="1" selected="0">
+            <x v="3"/>
+          </reference>
+        </references>
+      </pivotArea>
+    </chartFormat>
+    <chartFormat chart="2" format="12">
+      <pivotArea type="data" outline="0" fieldPosition="0">
+        <references count="3">
+          <reference field="4294967294" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="2" count="1" selected="0">
+            <x v="0"/>
+          </reference>
+          <reference field="11" count="1" selected="0">
+            <x v="2"/>
           </reference>
         </references>
       </pivotArea>
@@ -13269,9 +13989,9 @@
 
 <file path=xl/slicers/slicer1.xml><?xml version="1.0" encoding="utf-8"?>
 <slicers xmlns="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x xr10">
-  <slicer name="category" xr10:uid="{64E1BC70-1A9B-4CD9-B896-DA31F851DF95}" cache="Slicer_category" caption="Category" columnCount="2" style="SlicerStyleDark3" rowHeight="360000"/>
+  <slicer name="category" xr10:uid="{64E1BC70-1A9B-4CD9-B896-DA31F851DF95}" cache="Slicer_category" caption="Category" columnCount="2" style="SlicerStyleLight5" rowHeight="360000"/>
   <slicer name="region" xr10:uid="{4165D014-483A-412A-840E-6DC1DC07794D}" cache="Slicer_region" caption="Region" columnCount="4" style="SlicerStyleDark3" rowHeight="468000"/>
-  <slicer name="salesperson" xr10:uid="{04B5DD92-7045-437F-9E8D-E96F23A5A8F0}" cache="Slicer_salesperson" caption="Salesperson" columnCount="5" style="SlicerStyleDark3" rowHeight="360000"/>
+  <slicer name="salesperson" xr10:uid="{04B5DD92-7045-437F-9E8D-E96F23A5A8F0}" cache="Slicer_salesperson" caption="Salesperson" columnCount="5" style="SlicerStyleLight5" rowHeight="360000"/>
   <slicer name="product" xr10:uid="{322D932B-7E00-434A-91C3-ADA3090113D1}" cache="Slicer_product" caption="Product" columnCount="5" style="SlicerStyleDark3" rowHeight="360000"/>
 </slicers>
 </file>
@@ -15852,7 +16572,7 @@
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" scale="39" orientation="landscape" r:id="rId1"/>
+  <pageSetup paperSize="9" scale="38" orientation="landscape" r:id="rId1"/>
   <drawing r:id="rId2"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{A8765BA9-456A-4dab-B4F3-ACF838C121DE}">

</xml_diff>